<commit_message>
For Scientific Data (min rule revised)
</commit_message>
<xml_diff>
--- a/outputs_processed_data/p1_b_ember_2024_30_50.xlsx
+++ b/outputs_processed_data/p1_b_ember_2024_30_50.xlsx
@@ -1875,16 +1875,16 @@
         <v>89.49593836999999</v>
       </c>
       <c r="AC2">
-        <v>2708167.178239524</v>
+        <v>2503960.545795653</v>
       </c>
       <c r="AD2">
-        <v>1275141.861939513</v>
+        <v>1178991.067554601</v>
       </c>
       <c r="AE2">
-        <v>1793011.937346649</v>
+        <v>2141860.438846151</v>
       </c>
       <c r="AF2">
-        <v>643083.6025705481</v>
+        <v>594592.5278998286</v>
       </c>
       <c r="AG2">
         <v>0</v>
@@ -1893,16 +1893,16 @@
         <v>753440.0171152165</v>
       </c>
       <c r="AI2">
-        <v>2795808.629377285</v>
+        <v>2584993.481128652</v>
       </c>
       <c r="AJ2">
-        <v>1316407.88276897</v>
+        <v>1217145.465432694</v>
       </c>
       <c r="AK2">
-        <v>1851037.220777838</v>
+        <v>2211175.124624548</v>
       </c>
       <c r="AL2">
-        <v>663895.0135443788</v>
+        <v>613834.6752825786</v>
       </c>
       <c r="AM2">
         <v>0</v>
@@ -2205,10 +2205,10 @@
         <v>0</v>
       </c>
       <c r="AC5">
-        <v>8675436.507936507</v>
+        <v>8710000</v>
       </c>
       <c r="AD5">
-        <v>700000.0000000001</v>
+        <v>700000</v>
       </c>
       <c r="AE5">
         <v>1192441.314744938</v>
@@ -2223,13 +2223,13 @@
         <v>582788.9628365688</v>
       </c>
       <c r="AI5">
-        <v>9603916.688964158</v>
+        <v>9642179.305254852</v>
       </c>
       <c r="AJ5">
         <v>3404710.264440781</v>
       </c>
       <c r="AK5">
-        <v>3091463.756047942</v>
+        <v>3091463.756047941</v>
       </c>
       <c r="AL5">
         <v>0</v>
@@ -2330,13 +2330,13 @@
         <v>0</v>
       </c>
       <c r="AD6">
-        <v>22174455.21681652</v>
+        <v>80950961.23415618</v>
       </c>
       <c r="AE6">
-        <v>263916.5794116381</v>
+        <v>963464.5171711139</v>
       </c>
       <c r="AF6">
-        <v>6429007.874467505</v>
+        <v>23469995.63828833</v>
       </c>
       <c r="AG6">
         <v>48228708.62525191</v>
@@ -2449,16 +2449,16 @@
         <v>0</v>
       </c>
       <c r="AC7">
-        <v>42618375</v>
+        <v>53690843.93020726</v>
       </c>
       <c r="AD7">
-        <v>4278245.402298851</v>
+        <v>5389755.151151455</v>
       </c>
       <c r="AE7">
-        <v>0</v>
+        <v>22003089.18313745</v>
       </c>
       <c r="AF7">
-        <v>0</v>
+        <v>3313287.274243683</v>
       </c>
       <c r="AG7">
         <v>12280462.37113349</v>
@@ -2467,16 +2467,16 @@
         <v>81412824.88552621</v>
       </c>
       <c r="AI7">
-        <v>123078942.5909536</v>
+        <v>70932082.10018615</v>
       </c>
       <c r="AJ7">
-        <v>54284723.98842385</v>
+        <v>31285030.71016667</v>
       </c>
       <c r="AK7">
-        <v>0</v>
+        <v>68076345.37418057</v>
       </c>
       <c r="AL7">
-        <v>0</v>
+        <v>7070208.394844092</v>
       </c>
       <c r="AM7">
         <v>20519271.32827651</v>
@@ -2883,16 +2883,16 @@
         <v>0</v>
       </c>
       <c r="AC11">
-        <v>9940841.865756545</v>
+        <v>65757989.14810269</v>
       </c>
       <c r="AD11">
-        <v>81834338.44554201</v>
+        <v>418775217.0773629</v>
       </c>
       <c r="AE11">
-        <v>87577894.04839765</v>
+        <v>448167019.9570598</v>
       </c>
       <c r="AF11">
-        <v>0</v>
+        <v>15300886.19088148</v>
       </c>
       <c r="AG11">
         <v>0</v>
@@ -2901,16 +2901,16 @@
         <v>165983743.529539</v>
       </c>
       <c r="AI11">
-        <v>11878861.3768758</v>
+        <v>95174905.786488</v>
       </c>
       <c r="AJ11">
-        <v>429647507.3818066</v>
+        <v>227791657.5627147</v>
       </c>
       <c r="AK11">
-        <v>245084724.0561376</v>
+        <v>648655082.8821224</v>
       </c>
       <c r="AL11">
-        <v>0</v>
+        <v>22145756.28806219</v>
       </c>
       <c r="AM11">
         <v>0</v>
@@ -3005,16 +3005,16 @@
         <v>930</v>
       </c>
       <c r="AC12">
-        <v>44462986.06502987</v>
+        <v>53093299.98186032</v>
       </c>
       <c r="AD12">
-        <v>13001179.24528301</v>
+        <v>15421704.865678</v>
       </c>
       <c r="AE12">
-        <v>17099751.86104218</v>
+        <v>20283339.03426467</v>
       </c>
       <c r="AF12">
-        <v>4336681.234225745</v>
+        <v>7024702.150344338</v>
       </c>
       <c r="AG12">
         <v>0</v>
@@ -3023,16 +3023,16 @@
         <v>9477004.552629951</v>
       </c>
       <c r="AI12">
-        <v>52222436.42928072</v>
+        <v>54541141.38222929</v>
       </c>
       <c r="AJ12">
-        <v>14225134.90715485</v>
+        <v>15842251.01324142</v>
       </c>
       <c r="AK12">
-        <v>9972601.856475947</v>
+        <v>20836460.76528463</v>
       </c>
       <c r="AL12">
-        <v>5093496.413785148</v>
+        <v>7216264.072507856</v>
       </c>
       <c r="AM12">
         <v>0</v>
@@ -3335,16 +3335,16 @@
         <v>900</v>
       </c>
       <c r="AC15">
-        <v>519230.7692307693</v>
+        <v>9493963.306638448</v>
       </c>
       <c r="AD15">
-        <v>10624410.25641026</v>
+        <v>22277962.87253513</v>
       </c>
       <c r="AE15">
-        <v>27908571.42857143</v>
+        <v>58520529.90292591</v>
       </c>
       <c r="AF15">
-        <v>4436580.251317231</v>
+        <v>9302913.548564618</v>
       </c>
       <c r="AG15">
         <v>38284764.67859285</v>
@@ -3353,16 +3353,16 @@
         <v>15577145.41409291</v>
       </c>
       <c r="AI15">
-        <v>728243.0861647353</v>
+        <v>9493963.306638448</v>
       </c>
       <c r="AJ15">
-        <v>65470529.56644756</v>
+        <v>62037938.94223779</v>
       </c>
       <c r="AK15">
-        <v>91669244.58066976</v>
+        <v>86863067.02933896</v>
       </c>
       <c r="AL15">
-        <v>10050668.20219455</v>
+        <v>9523716.157261398</v>
       </c>
       <c r="AM15">
         <v>63969535.54662901</v>
@@ -3665,16 +3665,16 @@
         <v>0</v>
       </c>
       <c r="AC18">
-        <v>1547826.086956521</v>
+        <v>880169.9266032258</v>
       </c>
       <c r="AD18">
-        <v>5011764.705882354</v>
+        <v>2849935.538948582</v>
       </c>
       <c r="AE18">
-        <v>4372284.820731441</v>
+        <v>2486295.871468725</v>
       </c>
       <c r="AF18">
-        <v>0</v>
+        <v>247036.2873733965</v>
       </c>
       <c r="AG18">
         <v>0</v>
@@ -3683,16 +3683,16 @@
         <v>101260522.7821716</v>
       </c>
       <c r="AI18">
-        <v>7492688.131150017</v>
+        <v>7340334.383980061</v>
       </c>
       <c r="AJ18">
-        <v>106593626.8717267</v>
+        <v>104426188.6714327</v>
       </c>
       <c r="AK18">
-        <v>49567159.9340803</v>
+        <v>48559278.32732638</v>
       </c>
       <c r="AL18">
-        <v>0</v>
+        <v>3327673.554217864</v>
       </c>
       <c r="AM18">
         <v>0</v>
@@ -3787,16 +3787,16 @@
         <v>300</v>
       </c>
       <c r="AC19">
-        <v>2911646.586345383</v>
+        <v>3091799.289119156</v>
       </c>
       <c r="AD19">
-        <v>7511508.951406652</v>
+        <v>7719966.666675536</v>
       </c>
       <c r="AE19">
-        <v>5534285.714285713</v>
+        <v>5687871.972800279</v>
       </c>
       <c r="AF19">
-        <v>6825000</v>
+        <v>7014405.87249699</v>
       </c>
       <c r="AG19">
         <v>18734545.39405467</v>
@@ -3805,16 +3805,16 @@
         <v>8959581.89027372</v>
       </c>
       <c r="AI19">
-        <v>4099267.721163959</v>
+        <v>4228539.298876299</v>
       </c>
       <c r="AJ19">
-        <v>46464351.93268593</v>
+        <v>46389487.54743807</v>
       </c>
       <c r="AK19">
-        <v>18247328.72475598</v>
+        <v>18217928.22758831</v>
       </c>
       <c r="AL19">
-        <v>15520329.02023518</v>
+        <v>15495322.32493836</v>
       </c>
       <c r="AM19">
         <v>31303318.11089934</v>
@@ -4117,16 +4117,16 @@
         <v>25</v>
       </c>
       <c r="AC22">
-        <v>6608037.433155081</v>
+        <v>7229931.318632829</v>
       </c>
       <c r="AD22">
-        <v>2415619.047619048</v>
+        <v>2642957.153759375</v>
       </c>
       <c r="AE22">
-        <v>709090.9090909092</v>
+        <v>775824.6867173691</v>
       </c>
       <c r="AF22">
-        <v>100000</v>
+        <v>109411.1737678341</v>
       </c>
       <c r="AG22">
         <v>0</v>
@@ -4135,16 +4135,16 @@
         <v>8560167.905296978</v>
       </c>
       <c r="AI22">
-        <v>6608037.433155081</v>
+        <v>7229931.318632829</v>
       </c>
       <c r="AJ22">
-        <v>6167691.368138067</v>
+        <v>5636922.145728651</v>
       </c>
       <c r="AK22">
-        <v>965030.7011529466</v>
+        <v>881983.6476803613</v>
       </c>
       <c r="AL22">
-        <v>93864.15201831431</v>
+        <v>85786.54242256701</v>
       </c>
       <c r="AM22">
         <v>0</v>
@@ -4655,16 +4655,16 @@
         <v>23830</v>
       </c>
       <c r="AC27">
-        <v>431695117.2940535</v>
+        <v>413210000</v>
       </c>
       <c r="AD27">
-        <v>78558086.98926759</v>
+        <v>71320000</v>
       </c>
       <c r="AE27">
-        <v>125408646.8446602</v>
+        <v>111134443.75</v>
       </c>
       <c r="AF27">
-        <v>78013445.75604275</v>
+        <v>58240000.00000001</v>
       </c>
       <c r="AG27">
         <v>18407345.48162257</v>
@@ -4673,16 +4673,16 @@
         <v>71422482.58629547</v>
       </c>
       <c r="AI27">
-        <v>436137362.042575</v>
+        <v>417850689.8568216</v>
       </c>
       <c r="AJ27">
-        <v>79366468.26438928</v>
+        <v>72120982.55266938</v>
       </c>
       <c r="AK27">
-        <v>126699131.4495287</v>
+        <v>112382575.416354</v>
       </c>
       <c r="AL27">
-        <v>78816222.54419853</v>
+        <v>58894083.34082256</v>
       </c>
       <c r="AM27">
         <v>30756603.86033788</v>
@@ -5092,10 +5092,10 @@
         <v>0</v>
       </c>
       <c r="AD31">
-        <v>400000</v>
+        <v>755324.6714475943</v>
       </c>
       <c r="AE31">
-        <v>198740.2191241564</v>
+        <v>375283.4767834408</v>
       </c>
       <c r="AF31">
         <v>0</v>
@@ -5113,7 +5113,7 @@
         <v>3000438.115617846</v>
       </c>
       <c r="AK31">
-        <v>794612.6440016157</v>
+        <v>794612.6440016156</v>
       </c>
       <c r="AL31">
         <v>0</v>
@@ -5315,16 +5315,16 @@
         <v>2849.978453422537</v>
       </c>
       <c r="AC33">
-        <v>367021615.4651462</v>
+        <v>547252333.6555562</v>
       </c>
       <c r="AD33">
-        <v>9289512.521135842</v>
+        <v>14045813.0143152</v>
       </c>
       <c r="AE33">
-        <v>68048005.73619695</v>
+        <v>101463860.3575022</v>
       </c>
       <c r="AF33">
-        <v>10527646.25142261</v>
+        <v>15697383.30449452</v>
       </c>
       <c r="AG33">
         <v>125951675.4889643</v>
@@ -5333,16 +5333,16 @@
         <v>132687539.6099245</v>
       </c>
       <c r="AI33">
-        <v>505199405.7179652</v>
+        <v>547252333.6555562</v>
       </c>
       <c r="AJ33">
-        <v>56180963.71225618</v>
+        <v>48827229.56527273</v>
       </c>
       <c r="AK33">
-        <v>219359620.8288053</v>
+        <v>188005955.6344757</v>
       </c>
       <c r="AL33">
-        <v>23406318.84033043</v>
+        <v>20060790.24405252</v>
       </c>
       <c r="AM33">
         <v>210451082.8260084</v>
@@ -5437,16 +5437,16 @@
         <v>400</v>
       </c>
       <c r="AC34">
-        <v>47156781.75092478</v>
+        <v>112187325.347361</v>
       </c>
       <c r="AD34">
-        <v>7233632.862644415</v>
+        <v>17209018.36964174</v>
       </c>
       <c r="AE34">
-        <v>540000</v>
+        <v>1284675.362444276</v>
       </c>
       <c r="AF34">
-        <v>8555110.642781876</v>
+        <v>24143570.21438099</v>
       </c>
       <c r="AG34">
         <v>29272805.60354632</v>
@@ -5455,16 +5455,16 @@
         <v>1343483.404012675</v>
       </c>
       <c r="AI34">
-        <v>126523049.7056854</v>
+        <v>123151997.2632788</v>
       </c>
       <c r="AJ34">
-        <v>85272113.50787441</v>
+        <v>83000141.98032615</v>
       </c>
       <c r="AK34">
-        <v>3393042.886298896</v>
+        <v>3302639.394321306</v>
       </c>
       <c r="AL34">
-        <v>37075051.94978769</v>
+        <v>42808479.41172021</v>
       </c>
       <c r="AM34">
         <v>48911565.58819531</v>
@@ -5559,16 +5559,16 @@
         <v>882.0799999999999</v>
       </c>
       <c r="AC35">
-        <v>28243889.75606469</v>
+        <v>61111610.837695</v>
       </c>
       <c r="AD35">
-        <v>25696759.67326697</v>
+        <v>55600357.82979454</v>
       </c>
       <c r="AE35">
-        <v>33722820.01580042</v>
+        <v>72966431.71157782</v>
       </c>
       <c r="AF35">
-        <v>7200776.05193119</v>
+        <v>18140155.12356615</v>
       </c>
       <c r="AG35">
         <v>0</v>
@@ -5577,16 +5577,16 @@
         <v>24391485.85528418</v>
       </c>
       <c r="AI35">
-        <v>28243889.75606469</v>
+        <v>63089299.03147313</v>
       </c>
       <c r="AJ35">
-        <v>67834641.7935966</v>
+        <v>57399691.37284032</v>
       </c>
       <c r="AK35">
-        <v>47450640.86346092</v>
+        <v>75327764.50186151</v>
       </c>
       <c r="AL35">
-        <v>6988082.934418276</v>
+        <v>18727205.11503933</v>
       </c>
       <c r="AM35">
         <v>0</v>
@@ -5681,16 +5681,16 @@
         <v>82000</v>
       </c>
       <c r="AC36">
-        <v>1948712987.012987</v>
+        <v>1354250000</v>
       </c>
       <c r="AD36">
         <v>839040000</v>
       </c>
       <c r="AE36">
-        <v>0</v>
+        <v>997040000</v>
       </c>
       <c r="AF36">
-        <v>893260188.0877746</v>
+        <v>386618260.1880878</v>
       </c>
       <c r="AG36">
         <v>526676893.2667356</v>
@@ -5699,16 +5699,16 @@
         <v>5727185509.559084</v>
       </c>
       <c r="AI36">
-        <v>3089036214.783803</v>
+        <v>1899260881.782562</v>
       </c>
       <c r="AJ36">
-        <v>5843631988.029505</v>
+        <v>5170035396.382122</v>
       </c>
       <c r="AK36">
-        <v>0</v>
+        <v>3274676908.251177</v>
       </c>
       <c r="AL36">
-        <v>2287092571.7183</v>
+        <v>875787588.1157469</v>
       </c>
       <c r="AM36">
         <v>880017848.5687089</v>
@@ -6097,16 +6097,16 @@
         <v>62.02077895833333</v>
       </c>
       <c r="AC40">
-        <v>2542184.655386988</v>
+        <v>2823887.507072441</v>
       </c>
       <c r="AD40">
-        <v>544061.5210041401</v>
+        <v>500712.8677356957</v>
       </c>
       <c r="AE40">
-        <v>939031.5875177506</v>
+        <v>864213.2937698378</v>
       </c>
       <c r="AF40">
-        <v>2052511.123749825</v>
+        <v>1888975.219080729</v>
       </c>
       <c r="AG40">
         <v>0</v>
@@ -6115,16 +6115,16 @@
         <v>3721812.132737816</v>
       </c>
       <c r="AI40">
-        <v>3002411.586046152</v>
+        <v>3335112.79401324</v>
       </c>
       <c r="AJ40">
-        <v>873704.9727862807</v>
+        <v>801016.9248336632</v>
       </c>
       <c r="AK40">
-        <v>803788.9328899763</v>
+        <v>736917.5628995235</v>
       </c>
       <c r="AL40">
-        <v>2424089.518979882</v>
+        <v>2230947.728955865</v>
       </c>
       <c r="AM40">
         <v>0</v>
@@ -6219,16 +6219,16 @@
         <v>0</v>
       </c>
       <c r="AC41">
-        <v>57685325.26475039</v>
+        <v>50840000</v>
       </c>
       <c r="AD41">
-        <v>2309352.517985611</v>
+        <v>8058254.676258993</v>
       </c>
       <c r="AE41">
-        <v>11924413.14744939</v>
+        <v>436831.0016348959</v>
       </c>
       <c r="AF41">
-        <v>0</v>
+        <v>2270000</v>
       </c>
       <c r="AG41">
         <v>0</v>
@@ -6237,16 +6237,16 @@
         <v>28313004.98051037</v>
       </c>
       <c r="AI41">
-        <v>63946953.45801272</v>
+        <v>57282509.91548032</v>
       </c>
       <c r="AJ41">
-        <v>2560028.175415531</v>
+        <v>9079407.029785041</v>
       </c>
       <c r="AK41">
-        <v>13218784.65717897</v>
+        <v>492186.7856518514</v>
       </c>
       <c r="AL41">
-        <v>0</v>
+        <v>2557657.307398512</v>
       </c>
       <c r="AM41">
         <v>0</v>
@@ -6549,16 +6549,16 @@
         <v>402</v>
       </c>
       <c r="AC44">
-        <v>8606127.65957447</v>
+        <v>8680000</v>
       </c>
       <c r="AD44">
-        <v>834285.7142857143</v>
+        <v>80000</v>
       </c>
       <c r="AE44">
-        <v>1798650</v>
+        <v>1306620</v>
       </c>
       <c r="AF44">
-        <v>1915411.764705882</v>
+        <v>1620000</v>
       </c>
       <c r="AG44">
         <v>0</v>
@@ -6567,16 +6567,16 @@
         <v>671741.7020063376</v>
       </c>
       <c r="AI44">
-        <v>8727303.690732565</v>
+        <v>8817566.683399031</v>
       </c>
       <c r="AJ44">
-        <v>846032.6271491982</v>
+        <v>81267.89569953024</v>
       </c>
       <c r="AK44">
-        <v>1823975.358519407</v>
+        <v>1327328.223486502</v>
       </c>
       <c r="AL44">
-        <v>1942381.152665445</v>
+        <v>1645674.887915487</v>
       </c>
       <c r="AM44">
         <v>0</v>
@@ -6882,13 +6882,13 @@
         <v>0</v>
       </c>
       <c r="AD47">
-        <v>1370541.666666667</v>
+        <v>1427448.632572106</v>
       </c>
       <c r="AE47">
-        <v>212500</v>
+        <v>221323.3218653737</v>
       </c>
       <c r="AF47">
-        <v>135000</v>
+        <v>140605.4044791786</v>
       </c>
       <c r="AG47">
         <v>0</v>
@@ -6903,7 +6903,7 @@
         <v>5726269.561591201</v>
       </c>
       <c r="AK47">
-        <v>473242.2428629083</v>
+        <v>473242.2428629082</v>
       </c>
       <c r="AL47">
         <v>207357.088630658</v>
@@ -7001,16 +7001,16 @@
         <v>1600</v>
       </c>
       <c r="AC48">
-        <v>2586696.428571429</v>
+        <v>27034761.69742214</v>
       </c>
       <c r="AD48">
-        <v>9711538.461538462</v>
+        <v>63760475.33555956</v>
       </c>
       <c r="AE48">
-        <v>2833333.333333333</v>
+        <v>18602066.07149658</v>
       </c>
       <c r="AF48">
-        <v>10146341.46341463</v>
+        <v>66615146.21873095</v>
       </c>
       <c r="AG48">
         <v>34703328.77555586</v>
@@ -7019,16 +7019,16 @@
         <v>27940823.76723658</v>
       </c>
       <c r="AI48">
-        <v>8326189.836545795</v>
+        <v>27034761.69742214</v>
       </c>
       <c r="AJ48">
-        <v>137345347.1083471</v>
+        <v>109157353.9522845</v>
       </c>
       <c r="AK48">
-        <v>21358394.91436691</v>
+        <v>16974917.04382994</v>
       </c>
       <c r="AL48">
-        <v>52752247.05300767</v>
+        <v>66615146.21873095</v>
       </c>
       <c r="AM48">
         <v>57985358.9889133</v>
@@ -7123,16 +7123,16 @@
         <v>8200</v>
       </c>
       <c r="AC49">
-        <v>20372602.73972603</v>
+        <v>28124120.19190761</v>
       </c>
       <c r="AD49">
-        <v>177206470.9806538</v>
+        <v>184386535.4312977</v>
       </c>
       <c r="AE49">
-        <v>276001785.2238396</v>
+        <v>287184845.2748257</v>
       </c>
       <c r="AF49">
-        <v>37091741.29353233</v>
+        <v>47301951.52761611</v>
       </c>
       <c r="AG49">
         <v>0</v>
@@ -7141,16 +7141,16 @@
         <v>182332484.1418824</v>
       </c>
       <c r="AI49">
-        <v>28845683.42370207</v>
+        <v>42399769.39897812</v>
       </c>
       <c r="AJ49">
-        <v>88790110.37539682</v>
+        <v>50601310.39422157</v>
       </c>
       <c r="AK49">
-        <v>390792488.4540579</v>
+        <v>432958298.1243797</v>
       </c>
       <c r="AL49">
-        <v>52518406.24667676</v>
+        <v>71312162.77014951</v>
       </c>
       <c r="AM49">
         <v>0</v>
@@ -7358,7 +7358,7 @@
         <v>36129566.92913385</v>
       </c>
       <c r="AF51">
-        <v>6838639.807704587</v>
+        <v>7694384.040326445</v>
       </c>
       <c r="AG51">
         <v>0</v>
@@ -7376,7 +7376,7 @@
         <v>112506083.9481773</v>
       </c>
       <c r="AL51">
-        <v>14687352.92891577</v>
+        <v>16525235.59488705</v>
       </c>
       <c r="AM51">
         <v>0</v>
@@ -7575,16 +7575,16 @@
         <v>1415</v>
       </c>
       <c r="AC53">
-        <v>26461.53846153845</v>
+        <v>26461.53846153846</v>
       </c>
       <c r="AD53">
-        <v>29457065.2173913</v>
+        <v>20458872.22811946</v>
       </c>
       <c r="AE53">
-        <v>10020000</v>
+        <v>6959209.894566389</v>
       </c>
       <c r="AF53">
-        <v>6597702.492279531</v>
+        <v>4582315.016534634</v>
       </c>
       <c r="AG53">
         <v>0</v>
@@ -7593,16 +7593,16 @@
         <v>86591136.42484398</v>
       </c>
       <c r="AI53">
-        <v>26461.53846153845</v>
+        <v>32594.08446784633</v>
       </c>
       <c r="AJ53">
-        <v>110725969.9639798</v>
+        <v>110721116.9233292</v>
       </c>
       <c r="AK53">
-        <v>20075795.50267576</v>
+        <v>20074915.59481225</v>
       </c>
       <c r="AL53">
-        <v>9117133.588664468</v>
+        <v>9116733.991172235</v>
       </c>
       <c r="AM53">
         <v>0</v>
@@ -7697,16 +7697,16 @@
         <v>1490</v>
       </c>
       <c r="AC54">
-        <v>10742011.32183908</v>
+        <v>39017395.15727036</v>
       </c>
       <c r="AD54">
-        <v>266666.6666666666</v>
+        <v>449252.8286134372</v>
       </c>
       <c r="AE54">
-        <v>182857.1428571429</v>
+        <v>308059.0824777856</v>
       </c>
       <c r="AF54">
-        <v>4842500</v>
+        <v>8158150.584602138</v>
       </c>
       <c r="AG54">
         <v>0</v>
@@ -7715,16 +7715,16 @@
         <v>8487547.180755753</v>
       </c>
       <c r="AI54">
-        <v>18494963.72634422</v>
+        <v>40922361.49777595</v>
       </c>
       <c r="AJ54">
-        <v>2017259.094426729</v>
+        <v>471186.9304015229</v>
       </c>
       <c r="AK54">
-        <v>737309.6260942806</v>
+        <v>323099.6094181872</v>
       </c>
       <c r="AL54">
-        <v>13466916.03117755</v>
+        <v>8556460.164260156</v>
       </c>
       <c r="AM54">
         <v>0</v>
@@ -7819,16 +7819,16 @@
         <v>0</v>
       </c>
       <c r="AC55">
-        <v>14755908.12720848</v>
+        <v>36497834.33713362</v>
       </c>
       <c r="AD55">
-        <v>16405405.40540541</v>
+        <v>40577764.75416947</v>
       </c>
       <c r="AE55">
-        <v>19536363.63636364</v>
+        <v>48321998.03651755</v>
       </c>
       <c r="AF55">
-        <v>0</v>
+        <v>1588675.700378815</v>
       </c>
       <c r="AG55">
         <v>0</v>
@@ -7837,16 +7837,16 @@
         <v>175361995.8103707</v>
       </c>
       <c r="AI55">
-        <v>31541530.80729562</v>
+        <v>36497834.33713362</v>
       </c>
       <c r="AJ55">
-        <v>154073824.6063196</v>
+        <v>149723746.537158</v>
       </c>
       <c r="AK55">
-        <v>97798152.61243732</v>
+        <v>95036946.41812809</v>
       </c>
       <c r="AL55">
-        <v>0</v>
+        <v>2154980.733632823</v>
       </c>
       <c r="AM55">
         <v>0</v>
@@ -8045,16 +8045,16 @@
         <v>6660</v>
       </c>
       <c r="AC57">
-        <v>28165455.08625818</v>
+        <v>51520933.31906847</v>
       </c>
       <c r="AD57">
-        <v>144791655.8693962</v>
+        <v>228617874.5695578</v>
       </c>
       <c r="AE57">
-        <v>128688981.4523735</v>
+        <v>203192658.0541395</v>
       </c>
       <c r="AF57">
-        <v>34341438.89462581</v>
+        <v>54223199.00002699</v>
       </c>
       <c r="AG57">
         <v>66534083.04027005</v>
@@ -8063,16 +8063,16 @@
         <v>59149580.13882832</v>
       </c>
       <c r="AI57">
-        <v>28165455.08625818</v>
+        <v>51520933.31906847</v>
       </c>
       <c r="AJ57">
-        <v>403955188.520771</v>
+        <v>349776792.9666787</v>
       </c>
       <c r="AK57">
-        <v>191370963.7258087</v>
+        <v>203192658.0541395</v>
       </c>
       <c r="AL57">
-        <v>35221976.00707594</v>
+        <v>54223199.00002699</v>
       </c>
       <c r="AM57">
         <v>111170969.0744625</v>
@@ -8167,10 +8167,10 @@
         <v>367</v>
       </c>
       <c r="AC58">
-        <v>16000</v>
+        <v>20000</v>
       </c>
       <c r="AD58">
-        <v>857142.8571428572</v>
+        <v>950000.0000000001</v>
       </c>
       <c r="AE58">
         <v>4701052.631578948</v>
@@ -8185,10 +8185,10 @@
         <v>2387406.319292794</v>
       </c>
       <c r="AI58">
-        <v>19042.02064695291</v>
+        <v>23802.52580869115</v>
       </c>
       <c r="AJ58">
-        <v>4481994.622485381</v>
+        <v>4967544.039921297</v>
       </c>
       <c r="AK58">
         <v>13102623.40504026</v>
@@ -8289,16 +8289,16 @@
         <v>2409.2</v>
       </c>
       <c r="AC59">
-        <v>60891542.62295082</v>
+        <v>17620000</v>
       </c>
       <c r="AD59">
-        <v>4818400</v>
+        <v>40000</v>
       </c>
       <c r="AE59">
-        <v>4216100</v>
+        <v>987000</v>
       </c>
       <c r="AF59">
-        <v>301150</v>
+        <v>40000</v>
       </c>
       <c r="AG59">
         <v>0</v>
@@ -8307,16 +8307,16 @@
         <v>582788.9628365688</v>
       </c>
       <c r="AI59">
-        <v>61030872.14316869</v>
+        <v>17771515.75389301</v>
       </c>
       <c r="AJ59">
-        <v>4829425.264450514</v>
+        <v>40343.96311893987</v>
       </c>
       <c r="AK59">
-        <v>4225747.1063942</v>
+        <v>995487.2899598413</v>
       </c>
       <c r="AL59">
-        <v>301839.0790281571</v>
+        <v>40343.96311893987</v>
       </c>
       <c r="AM59">
         <v>0</v>
@@ -8411,16 +8411,16 @@
         <v>0</v>
       </c>
       <c r="AC60">
-        <v>14344827.5862069</v>
+        <v>19056974.24484457</v>
       </c>
       <c r="AD60">
-        <v>5945000</v>
+        <v>7897878.953563528</v>
       </c>
       <c r="AE60">
-        <v>24366028.70813397</v>
+        <v>32370049.67466712</v>
       </c>
       <c r="AF60">
-        <v>0</v>
+        <v>17087661.46900648</v>
       </c>
       <c r="AG60">
         <v>40135773.15463514</v>
@@ -8429,16 +8429,16 @@
         <v>4166614.070552824</v>
       </c>
       <c r="AI60">
-        <v>23000835.09843774</v>
+        <v>19056974.24484457</v>
       </c>
       <c r="AJ60">
-        <v>41881786.85912935</v>
+        <v>34502843.70122416</v>
       </c>
       <c r="AK60">
-        <v>91496213.06251298</v>
+        <v>75375951.58411096</v>
       </c>
       <c r="AL60">
-        <v>0</v>
+        <v>27443065.48990038</v>
       </c>
       <c r="AM60">
         <v>67062362.5105494</v>
@@ -8637,16 +8637,16 @@
         <v>0</v>
       </c>
       <c r="AC62">
-        <v>0</v>
+        <v>92513462.75153373</v>
       </c>
       <c r="AD62">
-        <v>59066418.95030191</v>
+        <v>78851932.89213912</v>
       </c>
       <c r="AE62">
-        <v>64001626.67751116</v>
+        <v>85440290.12507209</v>
       </c>
       <c r="AF62">
-        <v>0</v>
+        <v>13776896.61754442</v>
       </c>
       <c r="AG62">
         <v>473416832.3766375</v>
@@ -8655,16 +8655,16 @@
         <v>29093677.76932854</v>
       </c>
       <c r="AI62">
-        <v>0</v>
+        <v>253508978.6493201</v>
       </c>
       <c r="AJ62">
-        <v>1148699134.404046</v>
+        <v>949348840.0838726</v>
       </c>
       <c r="AK62">
-        <v>663440056.1022673</v>
+        <v>548303754.1006165</v>
       </c>
       <c r="AL62">
-        <v>0</v>
+        <v>60977617.67250426</v>
       </c>
       <c r="AM62">
         <v>791026277.4587051</v>
@@ -8967,16 +8967,16 @@
         <v>0</v>
       </c>
       <c r="AC65">
-        <v>10149698.63013699</v>
+        <v>13318248.72468045</v>
       </c>
       <c r="AD65">
-        <v>39496022.72727273</v>
+        <v>51825957.94081724</v>
       </c>
       <c r="AE65">
-        <v>212916504.8543689</v>
+        <v>279385139.6553085</v>
       </c>
       <c r="AF65">
-        <v>0</v>
+        <v>52618485.86064646</v>
       </c>
       <c r="AG65">
         <v>52614448.19875821</v>
@@ -8985,16 +8985,16 @@
         <v>88733447.79881014</v>
       </c>
       <c r="AI65">
-        <v>10149698.63013699</v>
+        <v>13318248.72468045</v>
       </c>
       <c r="AJ65">
-        <v>107768330.6865833</v>
+        <v>93365849.94575074</v>
       </c>
       <c r="AK65">
-        <v>309665016.1811089</v>
+        <v>268280460.9667515</v>
       </c>
       <c r="AL65">
-        <v>0</v>
+        <v>52618485.86064646</v>
       </c>
       <c r="AM65">
         <v>87912824.92063212</v>
@@ -9089,13 +9089,13 @@
         <v>0</v>
       </c>
       <c r="AC66">
-        <v>13275448.6803519</v>
+        <v>11340000</v>
       </c>
       <c r="AD66">
-        <v>1002114.013194145</v>
+        <v>393228.4125968924</v>
       </c>
       <c r="AE66">
-        <v>3375000</v>
+        <v>1324346.207158962</v>
       </c>
       <c r="AF66">
         <v>0</v>
@@ -9107,13 +9107,13 @@
         <v>2568958.130645859</v>
       </c>
       <c r="AI66">
-        <v>13808143.68723957</v>
+        <v>11955159.47641407</v>
       </c>
       <c r="AJ66">
-        <v>1042325.168689835</v>
+        <v>414559.8221563493</v>
       </c>
       <c r="AK66">
-        <v>3510426.35669307</v>
+        <v>1396187.840261861</v>
       </c>
       <c r="AL66">
         <v>0</v>
@@ -9211,16 +9211,16 @@
         <v>172.1</v>
       </c>
       <c r="AC67">
-        <v>872642.8481012657</v>
+        <v>18838618.30882299</v>
       </c>
       <c r="AD67">
-        <v>594710.5263157896</v>
+        <v>1216020.988105606</v>
       </c>
       <c r="AE67">
-        <v>1299761.033071983</v>
+        <v>2657657.172353622</v>
       </c>
       <c r="AF67">
-        <v>344200</v>
+        <v>703795.2173116544</v>
       </c>
       <c r="AG67">
         <v>0</v>
@@ -9229,16 +9229,16 @@
         <v>14339144.67108751</v>
       </c>
       <c r="AI67">
-        <v>2854145.803588679</v>
+        <v>22249086.33432892</v>
       </c>
       <c r="AJ67">
-        <v>8546146.213181159</v>
+        <v>2153629.249051609</v>
       </c>
       <c r="AK67">
-        <v>9955732.759443711</v>
+        <v>2508845.125234317</v>
       </c>
       <c r="AL67">
-        <v>1818365.287871564</v>
+        <v>458228.1383602319</v>
       </c>
       <c r="AM67">
         <v>0</v>
@@ -9749,16 +9749,16 @@
         <v>1000</v>
       </c>
       <c r="AC72">
-        <v>3581395.348837209</v>
+        <v>8639022.472827146</v>
       </c>
       <c r="AD72">
-        <v>17207119.74110033</v>
+        <v>41506921.08992022</v>
       </c>
       <c r="AE72">
-        <v>23227611.94029851</v>
+        <v>56029519.78130468</v>
       </c>
       <c r="AF72">
-        <v>3823529.411764706</v>
+        <v>9223096.948644718</v>
       </c>
       <c r="AG72">
         <v>0</v>
@@ -9767,16 +9767,16 @@
         <v>26125305.65370594</v>
       </c>
       <c r="AI72">
-        <v>3581395.348837209</v>
+        <v>12672429.79450251</v>
       </c>
       <c r="AJ72">
-        <v>44300258.96508048</v>
+        <v>14211683.55112085</v>
       </c>
       <c r="AK72">
-        <v>31874814.81826033</v>
+        <v>82188714.99426877</v>
       </c>
       <c r="AL72">
-        <v>3823529.411764706</v>
+        <v>13529198.34821793</v>
       </c>
       <c r="AM72">
         <v>0</v>
@@ -10495,16 +10495,16 @@
         <v>272</v>
       </c>
       <c r="AC79">
-        <v>7419392.694063926</v>
+        <v>19571896.21418204</v>
       </c>
       <c r="AD79">
-        <v>960000</v>
+        <v>2532420.258688746</v>
       </c>
       <c r="AE79">
-        <v>5317764.705882353</v>
+        <v>14027932.36678799</v>
       </c>
       <c r="AF79">
-        <v>1678332.079527136</v>
+        <v>4427335.582293469</v>
       </c>
       <c r="AG79">
         <v>0</v>
@@ -10513,16 +10513,16 @@
         <v>11419890.67987044</v>
       </c>
       <c r="AI79">
-        <v>8132020.753552016</v>
+        <v>21091329.05320164</v>
       </c>
       <c r="AJ79">
-        <v>4623026.948227284</v>
+        <v>2729020.652495351</v>
       </c>
       <c r="AK79">
-        <v>13649895.7268198</v>
+        <v>15116968.4452748</v>
       </c>
       <c r="AL79">
-        <v>2971246.346484524</v>
+        <v>4771044.694557317</v>
       </c>
       <c r="AM79">
         <v>0</v>
@@ -10617,16 +10617,16 @@
         <v>400</v>
       </c>
       <c r="AC80">
-        <v>383333.3333333333</v>
+        <v>400785.1115477677</v>
       </c>
       <c r="AD80">
-        <v>14649350.64935065</v>
+        <v>15316282.5237453</v>
       </c>
       <c r="AE80">
-        <v>2303125</v>
+        <v>2407977.939217702</v>
       </c>
       <c r="AF80">
-        <v>1161904.761904762</v>
+        <v>1913313.271649778</v>
       </c>
       <c r="AG80">
         <v>18710635.07764424</v>
@@ -10635,16 +10635,16 @@
         <v>9086668.158220865</v>
       </c>
       <c r="AI80">
-        <v>449493.5240906652</v>
+        <v>442857.7254921371</v>
       </c>
       <c r="AJ80">
-        <v>75472771.73220965</v>
+        <v>74358579.67816213</v>
       </c>
       <c r="AK80">
-        <v>6324620.323887173</v>
+        <v>6231250.999453907</v>
       </c>
       <c r="AL80">
-        <v>2200635.070726205</v>
+        <v>3414832.247805531</v>
       </c>
       <c r="AM80">
         <v>31263366.66158552</v>
@@ -10739,16 +10739,16 @@
         <v>7252.000000000001</v>
       </c>
       <c r="AC81">
-        <v>19012285.31855955</v>
+        <v>64967871.53528072</v>
       </c>
       <c r="AD81">
-        <v>12449634.14634146</v>
+        <v>29638190.98133956</v>
       </c>
       <c r="AE81">
-        <v>8663666.666666666</v>
+        <v>20625136.79093051</v>
       </c>
       <c r="AF81">
-        <v>45221145.6628478</v>
+        <v>107655609.4577542</v>
       </c>
       <c r="AG81">
         <v>0</v>
@@ -10757,16 +10757,16 @@
         <v>287735891.7279482</v>
       </c>
       <c r="AI81">
-        <v>52927953.04129625</v>
+        <v>72385130.50735247</v>
       </c>
       <c r="AJ81">
-        <v>152276342.107556</v>
+        <v>145086661.2934279</v>
       </c>
       <c r="AK81">
-        <v>56483630.82185131</v>
+        <v>53816773.50697492</v>
       </c>
       <c r="AL81">
-        <v>203340075.5799015</v>
+        <v>193739436.2428496</v>
       </c>
       <c r="AM81">
         <v>0</v>
@@ -10861,16 +10861,16 @@
         <v>14960</v>
       </c>
       <c r="AC82">
-        <v>215801199.7474216</v>
+        <v>271205003.4912036</v>
       </c>
       <c r="AD82">
-        <v>447281192.236599</v>
+        <v>562114100.5891274</v>
       </c>
       <c r="AE82">
-        <v>186207832.2259136</v>
+        <v>234013971.4145483</v>
       </c>
       <c r="AF82">
-        <v>30453796.88929553</v>
+        <v>38272364.10802428</v>
       </c>
       <c r="AG82">
         <v>64275490.42488853</v>
@@ -10879,16 +10879,16 @@
         <v>1443843513.47789</v>
       </c>
       <c r="AI82">
-        <v>215801199.7474216</v>
+        <v>271205003.4912036</v>
       </c>
       <c r="AJ82">
-        <v>1890505761.719284</v>
+        <v>1846073696.255277</v>
       </c>
       <c r="AK82">
-        <v>419508086.8829705</v>
+        <v>409648497.3717949</v>
       </c>
       <c r="AL82">
-        <v>47319962.12580343</v>
+        <v>46207813.35720305</v>
       </c>
       <c r="AM82">
         <v>107397114.8583547</v>
@@ -10983,16 +10983,16 @@
         <v>220</v>
       </c>
       <c r="AC83">
-        <v>728333.3333333334</v>
+        <v>2029094.691852182</v>
       </c>
       <c r="AD83">
-        <v>5791044.776119403</v>
+        <v>8793149.076205179</v>
       </c>
       <c r="AE83">
-        <v>32506072.87449393</v>
+        <v>49357370.85751747</v>
       </c>
       <c r="AF83">
-        <v>2912532.317147048</v>
+        <v>4422402.492819415</v>
       </c>
       <c r="AG83">
         <v>0</v>
@@ -11001,16 +11001,16 @@
         <v>15370769.60900641</v>
       </c>
       <c r="AI83">
-        <v>728333.3333333334</v>
+        <v>2162211.226568802</v>
       </c>
       <c r="AJ83">
-        <v>10808934.0658119</v>
+        <v>9370013.989888744</v>
       </c>
       <c r="AK83">
-        <v>32339661.80728331</v>
+        <v>52595407.10967404</v>
       </c>
       <c r="AL83">
-        <v>2912532.317147048</v>
+        <v>4712529.364340083</v>
       </c>
       <c r="AM83">
         <v>0</v>
@@ -11087,16 +11087,16 @@
         <v>27</v>
       </c>
       <c r="AC84">
-        <v>19438662.98811545</v>
+        <v>22984856.13873115</v>
       </c>
       <c r="AD84">
-        <v>68580487.48976114</v>
+        <v>66313293.35935584</v>
       </c>
       <c r="AE84">
-        <v>23328070.17861715</v>
+        <v>22556870.29773938</v>
       </c>
       <c r="AF84">
-        <v>15360445.78418505</v>
+        <v>14852646.64485241</v>
       </c>
       <c r="AG84">
         <v>8573763.579843214</v>
@@ -11105,16 +11105,16 @@
         <v>334006223.4634735</v>
       </c>
       <c r="AI84">
-        <v>27772505.32171381</v>
+        <v>33598090.91858957</v>
       </c>
       <c r="AJ84">
-        <v>430501142.0017376</v>
+        <v>425891016.9923403</v>
       </c>
       <c r="AK84">
-        <v>78054433.78194657</v>
+        <v>77218569.10665372</v>
       </c>
       <c r="AL84">
-        <v>35447297.71145173</v>
+        <v>35067701.79926608</v>
       </c>
       <c r="AM84">
         <v>14325794.57373152</v>
@@ -11197,7 +11197,7 @@
         <v>30441418.85257576</v>
       </c>
       <c r="AE85">
-        <v>10354833.87947028</v>
+        <v>10354833.87947029</v>
       </c>
       <c r="AF85">
         <v>6818174.979413335</v>
@@ -11313,16 +11313,16 @@
         <v>729.8095238095239</v>
       </c>
       <c r="AC86">
-        <v>13025714.28571429</v>
+        <v>14100000</v>
       </c>
       <c r="AD86">
-        <v>18320.18305656572</v>
+        <v>18320.18305656686</v>
       </c>
       <c r="AE86">
         <v>0</v>
       </c>
       <c r="AF86">
-        <v>5552095.238095238</v>
+        <v>6010000</v>
       </c>
       <c r="AG86">
         <v>0</v>
@@ -11331,16 +11331,16 @@
         <v>757625.6516875395</v>
       </c>
       <c r="AI86">
-        <v>17972636.26402408</v>
+        <v>19454915.54353121</v>
       </c>
       <c r="AJ86">
-        <v>111061.9048032908</v>
+        <v>111061.9048032978</v>
       </c>
       <c r="AK86">
         <v>0</v>
       </c>
       <c r="AL86">
-        <v>12373648.90696774</v>
+        <v>13394156.03331559</v>
       </c>
       <c r="AM86">
         <v>0</v>
@@ -11435,16 +11435,16 @@
         <v>0</v>
       </c>
       <c r="AC87">
-        <v>2217291.09589254</v>
+        <v>2373961.01087184</v>
       </c>
       <c r="AD87">
-        <v>21465579.71014493</v>
+        <v>22982300.06968619</v>
       </c>
       <c r="AE87">
-        <v>1523529.411764706</v>
+        <v>1631179.338223079</v>
       </c>
       <c r="AF87">
-        <v>0</v>
+        <v>117772.4078176509</v>
       </c>
       <c r="AG87">
         <v>0</v>
@@ -11453,16 +11453,16 @@
         <v>63245496.5953971</v>
       </c>
       <c r="AI87">
-        <v>2264198.533680293</v>
+        <v>2373961.01087184</v>
       </c>
       <c r="AJ87">
-        <v>96307361.60320461</v>
+        <v>96027289.76530169</v>
       </c>
       <c r="AK87">
-        <v>3643449.301843315</v>
+        <v>3632853.771810235</v>
       </c>
       <c r="AL87">
-        <v>0</v>
+        <v>180904.8907444355</v>
       </c>
       <c r="AM87">
         <v>0</v>
@@ -11557,16 +11557,16 @@
         <v>4240</v>
       </c>
       <c r="AC88">
-        <v>55743637.3220875</v>
+        <v>72638088.03640702</v>
       </c>
       <c r="AD88">
-        <v>78730288.80866426</v>
+        <v>102591397.4104721</v>
       </c>
       <c r="AE88">
-        <v>48026466.51270209</v>
+        <v>62582042.90599687</v>
       </c>
       <c r="AF88">
-        <v>22080772.9468599</v>
+        <v>28772882.54368007</v>
       </c>
       <c r="AG88">
         <v>0</v>
@@ -11575,16 +11575,16 @@
         <v>121739567.1027972</v>
       </c>
       <c r="AI88">
-        <v>67472319.03684463</v>
+        <v>110812283.5700356</v>
       </c>
       <c r="AJ88">
-        <v>85817718.68326908</v>
+        <v>49973518.10663436</v>
       </c>
       <c r="AK88">
-        <v>58131424.97383091</v>
+        <v>95471387.97782828</v>
       </c>
       <c r="AL88">
-        <v>26726654.88694858</v>
+        <v>43894173.23263723</v>
       </c>
       <c r="AM88">
         <v>0</v>
@@ -11786,13 +11786,13 @@
         <v>0</v>
       </c>
       <c r="AD90">
-        <v>4225028.702640644</v>
+        <v>10370704.43666335</v>
       </c>
       <c r="AE90">
-        <v>2143130.501339457</v>
+        <v>5260502.250481408</v>
       </c>
       <c r="AF90">
-        <v>78658.32035769839</v>
+        <v>193073.7633579224</v>
       </c>
       <c r="AG90">
         <v>0</v>
@@ -11804,13 +11804,13 @@
         <v>0</v>
       </c>
       <c r="AJ90">
-        <v>19941563.14607694</v>
+        <v>19897016.88837926</v>
       </c>
       <c r="AK90">
-        <v>5391668.424306732</v>
+        <v>5379624.300719716</v>
       </c>
       <c r="AL90">
-        <v>136483.3820732214</v>
+        <v>193073.7633579224</v>
       </c>
       <c r="AM90">
         <v>0</v>
@@ -11905,16 +11905,16 @@
         <v>9500</v>
       </c>
       <c r="AC91">
-        <v>142891628.2369635</v>
+        <v>163873118.0188679</v>
       </c>
       <c r="AD91">
-        <v>124134046.5014736</v>
+        <v>142361267.0908977</v>
       </c>
       <c r="AE91">
-        <v>46714236.70668954</v>
+        <v>53573520.85247217</v>
       </c>
       <c r="AF91">
-        <v>77996916.111564</v>
+        <v>89449591.95133375</v>
       </c>
       <c r="AG91">
         <v>99047383.06999826</v>
@@ -11923,16 +11923,16 @@
         <v>633951692.4731973</v>
       </c>
       <c r="AI91">
-        <v>215629384.3350096</v>
+        <v>215629384.3350095</v>
       </c>
       <c r="AJ91">
-        <v>823032798.0160751</v>
+        <v>823032798.016075</v>
       </c>
       <c r="AK91">
         <v>165089902.539682</v>
       </c>
       <c r="AL91">
-        <v>190111870.2331442</v>
+        <v>190111870.2331441</v>
       </c>
       <c r="AM91">
         <v>165497036.3612984</v>
@@ -12131,13 +12131,13 @@
         <v>3670</v>
       </c>
       <c r="AC93">
-        <v>2812441.860465116</v>
+        <v>3610000</v>
       </c>
       <c r="AD93">
         <v>3968918.918918917</v>
       </c>
       <c r="AE93">
-        <v>8227272.727272728</v>
+        <v>8227272.727272727</v>
       </c>
       <c r="AF93">
         <v>18967079.6460177</v>
@@ -12149,16 +12149,16 @@
         <v>944069.4190359339</v>
       </c>
       <c r="AI93">
-        <v>4919313.550508633</v>
+        <v>6314342.766324515</v>
       </c>
       <c r="AJ93">
-        <v>30501292.98082309</v>
+        <v>30501292.98082308</v>
       </c>
       <c r="AK93">
-        <v>33701322.34498078</v>
+        <v>33701322.34498076</v>
       </c>
       <c r="AL93">
-        <v>53586089.3669671</v>
+        <v>53586089.36696708</v>
       </c>
       <c r="AM93">
         <v>0</v>
@@ -12357,16 +12357,16 @@
         <v>98</v>
       </c>
       <c r="AC95">
-        <v>6162238.805970149</v>
+        <v>5300000</v>
       </c>
       <c r="AD95">
-        <v>1221988.636363636</v>
+        <v>1070000</v>
       </c>
       <c r="AE95">
         <v>0</v>
       </c>
       <c r="AF95">
-        <v>42000.00000000001</v>
+        <v>30000</v>
       </c>
       <c r="AG95">
         <v>0</v>
@@ -12375,16 +12375,16 @@
         <v>8565404.976778315</v>
       </c>
       <c r="AI95">
-        <v>7354422.348246003</v>
+        <v>7300583.341870322</v>
       </c>
       <c r="AJ95">
-        <v>6407701.634452899</v>
+        <v>6475756.988787701</v>
       </c>
       <c r="AK95">
         <v>0</v>
       </c>
       <c r="AL95">
-        <v>80963.63109403747</v>
+        <v>66747.28313491624</v>
       </c>
       <c r="AM95">
         <v>0</v>
@@ -12687,16 +12687,16 @@
         <v>2108</v>
       </c>
       <c r="AC98">
-        <v>4560388.888888889</v>
+        <v>14620000</v>
       </c>
       <c r="AD98">
-        <v>77491764.35272045</v>
+        <v>73039624.1082136</v>
       </c>
       <c r="AE98">
-        <v>26706156.52173913</v>
+        <v>25171805.6753016</v>
       </c>
       <c r="AF98">
-        <v>15998776.11940298</v>
+        <v>20340000</v>
       </c>
       <c r="AG98">
         <v>228806151.3988032</v>
@@ -12705,16 +12705,16 @@
         <v>345628315.6482617</v>
       </c>
       <c r="AI98">
-        <v>14853709.80079742</v>
+        <v>48296842.34744761</v>
       </c>
       <c r="AJ98">
-        <v>1108954370.229219</v>
+        <v>1060119848.94395</v>
       </c>
       <c r="AK98">
-        <v>203711028.8298265</v>
+        <v>194740298.5270297</v>
       </c>
       <c r="AL98">
-        <v>84168669.42922546</v>
+        <v>108530788.470641</v>
       </c>
       <c r="AM98">
         <v>382309343.1047593</v>
@@ -12913,16 +12913,16 @@
         <v>112</v>
       </c>
       <c r="AC100">
-        <v>71492842.53578733</v>
+        <v>40000000</v>
       </c>
       <c r="AD100">
-        <v>2121333.333333333</v>
+        <v>90266.66666666667</v>
       </c>
       <c r="AE100">
-        <v>2384882.629489877</v>
+        <v>0</v>
       </c>
       <c r="AF100">
-        <v>37333.33333333333</v>
+        <v>40000</v>
       </c>
       <c r="AG100">
         <v>0</v>
@@ -12931,16 +12931,16 @@
         <v>11056505.31140161</v>
       </c>
       <c r="AI100">
-        <v>74359257.73493643</v>
+        <v>43038687.07705425</v>
       </c>
       <c r="AJ100">
-        <v>2206385.51329225</v>
+        <v>97123.97050388575</v>
       </c>
       <c r="AK100">
-        <v>2480501.485516401</v>
+        <v>0</v>
       </c>
       <c r="AL100">
-        <v>38830.16616730547</v>
+        <v>43038.68707705424</v>
       </c>
       <c r="AM100">
         <v>0</v>
@@ -13017,16 +13017,16 @@
         <v>50.10275</v>
       </c>
       <c r="AC101">
-        <v>700000</v>
+        <v>783828.7967110248</v>
       </c>
       <c r="AD101">
-        <v>2152374.959876992</v>
+        <v>2099316.380721157</v>
       </c>
       <c r="AE101">
-        <v>1393965.01418051</v>
+        <v>1359602.133909133</v>
       </c>
       <c r="AF101">
-        <v>30000</v>
+        <v>33592.66271618678</v>
       </c>
       <c r="AG101">
         <v>0</v>
@@ -13035,16 +13035,16 @@
         <v>4258800.260874717</v>
       </c>
       <c r="AI101">
-        <v>700000</v>
+        <v>783828.7967110248</v>
       </c>
       <c r="AJ101">
-        <v>4573954.934667153</v>
+        <v>4508967.544794073</v>
       </c>
       <c r="AK101">
-        <v>1578958.984845793</v>
+        <v>1556524.915291662</v>
       </c>
       <c r="AL101">
-        <v>30000</v>
+        <v>33592.66271618678</v>
       </c>
       <c r="AM101">
         <v>0</v>
@@ -13451,16 +13451,16 @@
         <v>220</v>
       </c>
       <c r="AC105">
-        <v>8358535.135135137</v>
+        <v>9195893.656793786</v>
       </c>
       <c r="AD105">
-        <v>4144903.448275862</v>
+        <v>4560140.109694765</v>
       </c>
       <c r="AE105">
-        <v>5998592.592592591</v>
+        <v>6599531.937125795</v>
       </c>
       <c r="AF105">
-        <v>770000</v>
+        <v>847138.643464796</v>
       </c>
       <c r="AG105">
         <v>0</v>
@@ -13469,16 +13469,16 @@
         <v>9086873.291605348</v>
       </c>
       <c r="AI105">
-        <v>11853473.02132431</v>
+        <v>10282562.73559902</v>
       </c>
       <c r="AJ105">
-        <v>325328.4959706991</v>
+        <v>5099007.068923232</v>
       </c>
       <c r="AK105">
-        <v>8506772.336617399</v>
+        <v>7379391.683042279</v>
       </c>
       <c r="AL105">
-        <v>1091958.588300192</v>
+        <v>947244.1257236204</v>
       </c>
       <c r="AM105">
         <v>0</v>
@@ -13558,13 +13558,13 @@
         <v>480000</v>
       </c>
       <c r="AD106">
-        <v>35737.30040332724</v>
+        <v>63757.14717975852</v>
       </c>
       <c r="AE106">
-        <v>61681.35888272046</v>
+        <v>110042.6566122766</v>
       </c>
       <c r="AF106">
-        <v>134821.5298800006</v>
+        <v>240528.4122344931</v>
       </c>
       <c r="AG106">
         <v>0</v>
@@ -13576,13 +13576,13 @@
         <v>760657.2000073725</v>
       </c>
       <c r="AJ106">
-        <v>248825.3121461066</v>
+        <v>443916.9122878586</v>
       </c>
       <c r="AK106">
-        <v>228913.6932437462</v>
+        <v>408393.5794502484</v>
       </c>
       <c r="AL106">
-        <v>345094.182986332</v>
+        <v>615665.435475636</v>
       </c>
       <c r="AM106">
         <v>0</v>
@@ -13677,7 +13677,7 @@
         <v>0</v>
       </c>
       <c r="AC107">
-        <v>4190111.111111111</v>
+        <v>4782555.555555555</v>
       </c>
       <c r="AD107">
         <v>2798054.474708171</v>
@@ -13686,7 +13686,7 @@
         <v>24109005.46448088</v>
       </c>
       <c r="AF107">
-        <v>0</v>
+        <v>999934.0468677902</v>
       </c>
       <c r="AG107">
         <v>0</v>
@@ -13695,7 +13695,7 @@
         <v>689896.8831416441</v>
       </c>
       <c r="AI107">
-        <v>4617508.284062897</v>
+        <v>5270382.887510788</v>
       </c>
       <c r="AJ107">
         <v>13547631.67760056</v>
@@ -13704,7 +13704,7 @@
         <v>62220218.99774873</v>
       </c>
       <c r="AL107">
-        <v>0</v>
+        <v>1779853.038998933</v>
       </c>
       <c r="AM107">
         <v>0</v>
@@ -13799,16 +13799,16 @@
         <v>120</v>
       </c>
       <c r="AC108">
-        <v>186666.6666666667</v>
+        <v>6038666.666666667</v>
       </c>
       <c r="AD108">
-        <v>834615.3846153846</v>
+        <v>350000</v>
       </c>
       <c r="AE108">
-        <v>964285.7142857144</v>
+        <v>449999.9999999999</v>
       </c>
       <c r="AF108">
-        <v>598433.1553934015</v>
+        <v>498694.296161168</v>
       </c>
       <c r="AG108">
         <v>0</v>
@@ -13817,16 +13817,16 @@
         <v>136163.8585147982</v>
       </c>
       <c r="AI108">
-        <v>189378.8316976496</v>
+        <v>6069565.577881244</v>
       </c>
       <c r="AJ108">
-        <v>846741.8917250681</v>
+        <v>351790.8951631324</v>
       </c>
       <c r="AK108">
-        <v>978296.2606830116</v>
+        <v>452302.5794954558</v>
       </c>
       <c r="AL108">
-        <v>607128.0633082521</v>
+        <v>501246.0367408158</v>
       </c>
       <c r="AM108">
         <v>0</v>
@@ -13921,16 +13921,16 @@
         <v>140</v>
       </c>
       <c r="AC109">
-        <v>3393081.761006289</v>
+        <v>13144990.15070698</v>
       </c>
       <c r="AD109">
-        <v>1736170.212765957</v>
+        <v>6726021.344086632</v>
       </c>
       <c r="AE109">
-        <v>2720769.230769231</v>
+        <v>10540413.48246246</v>
       </c>
       <c r="AF109">
-        <v>861538.4615384616</v>
+        <v>3337648.60061011</v>
       </c>
       <c r="AG109">
         <v>0</v>
@@ -13939,16 +13939,16 @@
         <v>1590270.48272668</v>
       </c>
       <c r="AI109">
-        <v>4415267.314837615</v>
+        <v>13315775.08679609</v>
       </c>
       <c r="AJ109">
-        <v>9926132.089105971</v>
+        <v>6813408.486428614</v>
       </c>
       <c r="AK109">
-        <v>8291335.358662003</v>
+        <v>10677358.72337299</v>
       </c>
       <c r="AL109">
-        <v>1810789.604968244</v>
+        <v>3381012.657669706</v>
       </c>
       <c r="AM109">
         <v>0</v>
@@ -14147,16 +14147,16 @@
         <v>0</v>
       </c>
       <c r="AC111">
-        <v>808091.6030534351</v>
+        <v>1020025.383163633</v>
       </c>
       <c r="AD111">
-        <v>6069354.838709679</v>
+        <v>7661131.45034316</v>
       </c>
       <c r="AE111">
-        <v>16382253.52112676</v>
+        <v>20678737.85822043</v>
       </c>
       <c r="AF111">
-        <v>0</v>
+        <v>50490.58197409257</v>
       </c>
       <c r="AG111">
         <v>0</v>
@@ -14165,16 +14165,16 @@
         <v>29289756.48239255</v>
       </c>
       <c r="AI111">
-        <v>808091.6030534351</v>
+        <v>1020025.383163633</v>
       </c>
       <c r="AJ111">
-        <v>19079241.52715588</v>
+        <v>18971634.08844038</v>
       </c>
       <c r="AK111">
-        <v>27449677.35226814</v>
+        <v>27294860.42889935</v>
       </c>
       <c r="AL111">
-        <v>0</v>
+        <v>50490.58197409257</v>
       </c>
       <c r="AM111">
         <v>0</v>
@@ -14269,16 +14269,16 @@
         <v>98</v>
       </c>
       <c r="AC112">
-        <v>88000</v>
+        <v>715696.9841852764</v>
       </c>
       <c r="AD112">
-        <v>94852.94117647059</v>
+        <v>447310.6151157978</v>
       </c>
       <c r="AE112">
-        <v>1050000</v>
+        <v>3131174.305810585</v>
       </c>
       <c r="AF112">
-        <v>98000</v>
+        <v>292242.9352089879</v>
       </c>
       <c r="AG112">
         <v>0</v>
@@ -14287,16 +14287,16 @@
         <v>8863501.377628464</v>
       </c>
       <c r="AI112">
-        <v>403769.6854969042</v>
+        <v>977710.7552372657</v>
       </c>
       <c r="AJ112">
-        <v>1912171.808597188</v>
+        <v>2684821.899940657</v>
       </c>
       <c r="AK112">
-        <v>11282632.24679526</v>
+        <v>10017481.43429274</v>
       </c>
       <c r="AL112">
-        <v>726286.1423423956</v>
+        <v>644845.7937610799</v>
       </c>
       <c r="AM112">
         <v>0</v>
@@ -14599,16 +14599,16 @@
         <v>1036</v>
       </c>
       <c r="AC115">
-        <v>28059166.66666666</v>
+        <v>32804939.32352877</v>
       </c>
       <c r="AD115">
-        <v>30561537.94829025</v>
+        <v>35730547.87897182</v>
       </c>
       <c r="AE115">
-        <v>49634016.39344262</v>
+        <v>58028840.11178466</v>
       </c>
       <c r="AF115">
-        <v>4916973.274954378</v>
+        <v>10159934.46925522</v>
       </c>
       <c r="AG115">
         <v>14359595.87317959</v>
@@ -14617,16 +14617,16 @@
         <v>243161418.5357265</v>
       </c>
       <c r="AI115">
-        <v>43729462.09740817</v>
+        <v>42818668.43304251</v>
       </c>
       <c r="AJ115">
-        <v>209266467.6880911</v>
+        <v>204907882.7937713</v>
       </c>
       <c r="AK115">
-        <v>181154398.1803762</v>
+        <v>177381329.1733271</v>
       </c>
       <c r="AL115">
-        <v>12377355.33524819</v>
+        <v>21419802.90098282</v>
       </c>
       <c r="AM115">
         <v>23993269.55137891</v>
@@ -14721,16 +14721,16 @@
         <v>25.19</v>
       </c>
       <c r="AC116">
-        <v>2567251.267605634</v>
+        <v>4532601.369890139</v>
       </c>
       <c r="AD116">
-        <v>320489.6385542169</v>
+        <v>565839.3446237404</v>
       </c>
       <c r="AE116">
-        <v>820474.2857142856</v>
+        <v>1448585.465051361</v>
       </c>
       <c r="AF116">
-        <v>176330</v>
+        <v>311318.8060855996</v>
       </c>
       <c r="AG116">
         <v>0</v>
@@ -14739,16 +14739,16 @@
         <v>3533086.810789826</v>
       </c>
       <c r="AI116">
-        <v>2567251.267605634</v>
+        <v>6217407.74229029</v>
       </c>
       <c r="AJ116">
-        <v>1224384.365923448</v>
+        <v>502445.5420478924</v>
       </c>
       <c r="AK116">
-        <v>1670758.891986868</v>
+        <v>685622.4078641688</v>
       </c>
       <c r="AL116">
-        <v>247648.4206724268</v>
+        <v>427038.6467548748</v>
       </c>
       <c r="AM116">
         <v>0</v>
@@ -14950,7 +14950,7 @@
         <v>0</v>
       </c>
       <c r="AD118">
-        <v>422608.6956521739</v>
+        <v>1113517.776298794</v>
       </c>
       <c r="AE118">
         <v>0</v>
@@ -15069,16 +15069,16 @@
         <v>0</v>
       </c>
       <c r="AC119">
-        <v>21712079.51070336</v>
+        <v>9530000</v>
       </c>
       <c r="AD119">
-        <v>177272.7272727273</v>
+        <v>207350</v>
       </c>
       <c r="AE119">
-        <v>0</v>
+        <v>834708.9203214571</v>
       </c>
       <c r="AF119">
-        <v>0</v>
+        <v>270000</v>
       </c>
       <c r="AG119">
         <v>0</v>
@@ -15087,16 +15087,16 @@
         <v>13289592.5910443</v>
       </c>
       <c r="AI119">
-        <v>25346710.56165896</v>
+        <v>15951340.76949335</v>
       </c>
       <c r="AJ119">
-        <v>206948.4181118018</v>
+        <v>1524872.048658219</v>
       </c>
       <c r="AK119">
-        <v>0</v>
+        <v>3271970.981160932</v>
       </c>
       <c r="AL119">
-        <v>0</v>
+        <v>729959.3927722204</v>
       </c>
       <c r="AM119">
         <v>0</v>
@@ -15191,16 +15191,16 @@
         <v>39</v>
       </c>
       <c r="AC120">
-        <v>3256000</v>
+        <v>2501820.50976592</v>
       </c>
       <c r="AD120">
-        <v>840000.0000000001</v>
+        <v>645432.8096447705</v>
       </c>
       <c r="AE120">
-        <v>475000</v>
+        <v>364976.8864062689</v>
       </c>
       <c r="AF120">
-        <v>181844.8036741355</v>
+        <v>139724.5268508321</v>
       </c>
       <c r="AG120">
         <v>0</v>
@@ -15209,16 +15209,16 @@
         <v>1334405.813445022</v>
       </c>
       <c r="AI120">
-        <v>3508057.046178211</v>
+        <v>2753877.55594413</v>
       </c>
       <c r="AJ120">
-        <v>905027.0020852879</v>
+        <v>710459.8117300582</v>
       </c>
       <c r="AK120">
-        <v>511771.2214172758</v>
+        <v>401748.1078235447</v>
       </c>
       <c r="AL120">
-        <v>195921.9732309412</v>
+        <v>153801.6964076377</v>
       </c>
       <c r="AM120">
         <v>0</v>
@@ -15503,16 +15503,16 @@
         <v>62.02077895833333</v>
       </c>
       <c r="AC123">
-        <v>1070651.913980171</v>
+        <v>957643.1323067382</v>
       </c>
       <c r="AD123">
-        <v>229133.8308378602</v>
+        <v>293724.7021563826</v>
       </c>
       <c r="AE123">
-        <v>433333.3333333334</v>
+        <v>572992.3661514065</v>
       </c>
       <c r="AF123">
-        <v>864423.816913418</v>
+        <v>773182.6944502556</v>
       </c>
       <c r="AG123">
         <v>0</v>
@@ -15521,16 +15521,16 @@
         <v>1590638.773549632</v>
       </c>
       <c r="AI123">
-        <v>1264478.449409576</v>
+        <v>1131011.010408916</v>
       </c>
       <c r="AJ123">
-        <v>373862.8736124572</v>
+        <v>486299.6630390609</v>
       </c>
       <c r="AK123">
-        <v>376868.8529452553</v>
+        <v>505658.5524477884</v>
       </c>
       <c r="AL123">
-        <v>1020915.643423236</v>
+        <v>913156.5934947592</v>
       </c>
       <c r="AM123">
         <v>0</v>
@@ -15613,7 +15613,7 @@
         <v>279532.2276090384</v>
       </c>
       <c r="AE124">
-        <v>503206.5486339729</v>
+        <v>503206.5486339728</v>
       </c>
       <c r="AF124">
         <v>320000</v>
@@ -15625,7 +15625,7 @@
         <v>2477226.6891201</v>
       </c>
       <c r="AI124">
-        <v>119570.0120984971</v>
+        <v>119570.0120984972</v>
       </c>
       <c r="AJ124">
         <v>1631686.502037989</v>
@@ -15634,7 +15634,7 @@
         <v>1565655.27034058</v>
       </c>
       <c r="AL124">
-        <v>686689.4684334628</v>
+        <v>686689.4684334629</v>
       </c>
       <c r="AM124">
         <v>0</v>
@@ -15833,16 +15833,16 @@
         <v>490</v>
       </c>
       <c r="AC126">
-        <v>42044044.94382022</v>
+        <v>33828588.63997977</v>
       </c>
       <c r="AD126">
-        <v>12235151.51515152</v>
+        <v>9844388.38144478</v>
       </c>
       <c r="AE126">
         <v>0</v>
       </c>
       <c r="AF126">
-        <v>791538.4615384614</v>
+        <v>1470000</v>
       </c>
       <c r="AG126">
         <v>0</v>
@@ -15851,16 +15851,16 @@
         <v>144533397.0181744</v>
       </c>
       <c r="AI126">
-        <v>101165013.345202</v>
+        <v>99451655.21791553</v>
       </c>
       <c r="AJ126">
-        <v>129348165.9131776</v>
+        <v>127157490.263675</v>
       </c>
       <c r="AK126">
         <v>0</v>
       </c>
       <c r="AL126">
-        <v>3076298.818377931</v>
+        <v>6980332.595166999</v>
       </c>
       <c r="AM126">
         <v>0</v>
@@ -16041,16 +16041,16 @@
         <v>58.73</v>
       </c>
       <c r="AC128">
-        <v>834459.1261678346</v>
+        <v>1115145.837624968</v>
       </c>
       <c r="AD128">
-        <v>872211.6117639386</v>
+        <v>756230.7789330842</v>
       </c>
       <c r="AE128">
-        <v>787589.8896396178</v>
+        <v>682861.484172934</v>
       </c>
       <c r="AF128">
-        <v>451049.0850703883</v>
+        <v>391071.6119107935</v>
       </c>
       <c r="AG128">
         <v>0</v>
@@ -16059,16 +16059,16 @@
         <v>2069690.649424932</v>
       </c>
       <c r="AI128">
-        <v>877124.0410437159</v>
+        <v>1172161.934332973</v>
       </c>
       <c r="AJ128">
-        <v>1461374.241272133</v>
+        <v>1304760.083041285</v>
       </c>
       <c r="AK128">
-        <v>703371.4574692432</v>
+        <v>627991.7733171142</v>
       </c>
       <c r="AL128">
-        <v>474110.6949394637</v>
+        <v>411066.6440331839</v>
       </c>
       <c r="AM128">
         <v>0</v>
@@ -16267,16 +16267,16 @@
         <v>6474</v>
       </c>
       <c r="AC130">
-        <v>18731468.53146853</v>
+        <v>9080000</v>
       </c>
       <c r="AD130">
-        <v>4285714.285714286</v>
+        <v>648151.2474684035</v>
       </c>
       <c r="AE130">
-        <v>3179843.505986502</v>
+        <v>480904.5582038723</v>
       </c>
       <c r="AF130">
-        <v>19422000</v>
+        <v>2937291.82327731</v>
       </c>
       <c r="AG130">
         <v>0</v>
@@ -16285,16 +16285,16 @@
         <v>29261225.36766198</v>
       </c>
       <c r="AI130">
-        <v>21264962.40580774</v>
+        <v>24125917.87426234</v>
       </c>
       <c r="AJ130">
-        <v>10590337.76543967</v>
+        <v>7566576.539783902</v>
       </c>
       <c r="AK130">
-        <v>4188296.013050891</v>
+        <v>2992450.576736221</v>
       </c>
       <c r="AL130">
-        <v>17643555.97894776</v>
+        <v>12605954.56967729</v>
       </c>
       <c r="AM130">
         <v>0</v>
@@ -16493,16 +16493,16 @@
         <v>590</v>
       </c>
       <c r="AC132">
-        <v>100000</v>
+        <v>152801.0425197595</v>
       </c>
       <c r="AD132">
-        <v>24101143.45114345</v>
+        <v>36826798.45252994</v>
       </c>
       <c r="AE132">
-        <v>66858904.10958904</v>
+        <v>102161102.4967384</v>
       </c>
       <c r="AF132">
-        <v>7066126.352099644</v>
+        <v>37189655.18289231</v>
       </c>
       <c r="AG132">
         <v>4240564.939850425</v>
@@ -16511,16 +16511,16 @@
         <v>51442705.74689075</v>
       </c>
       <c r="AI132">
-        <v>100000</v>
+        <v>204212.6249183197</v>
       </c>
       <c r="AJ132">
-        <v>53761703.02420904</v>
+        <v>1228528.825749048</v>
       </c>
       <c r="AK132">
-        <v>79494969.69846497</v>
+        <v>136534323.0738141</v>
       </c>
       <c r="AL132">
-        <v>7066126.352099644</v>
+        <v>49702521.5238537</v>
       </c>
       <c r="AM132">
         <v>7085507.040068891</v>
@@ -16615,16 +16615,16 @@
         <v>190</v>
       </c>
       <c r="AC133">
-        <v>138460086.4553314</v>
+        <v>140143582.2340441</v>
       </c>
       <c r="AD133">
-        <v>2425500</v>
+        <v>2454283.456380317</v>
       </c>
       <c r="AE133">
-        <v>25818446.60194174</v>
+        <v>26124834.61743321</v>
       </c>
       <c r="AF133">
-        <v>866345.8135310945</v>
+        <v>876626.7564022727</v>
       </c>
       <c r="AG133">
         <v>0</v>
@@ -16633,16 +16633,16 @@
         <v>2251242.460777996</v>
       </c>
       <c r="AI133">
-        <v>138972982.9991936</v>
+        <v>140656504.4565071</v>
       </c>
       <c r="AJ133">
-        <v>2434484.759427685</v>
+        <v>2463266.07624013</v>
       </c>
       <c r="AK133">
-        <v>25914085.65843111</v>
+        <v>26220450.89910549</v>
       </c>
       <c r="AL133">
-        <v>869555.0111051034</v>
+        <v>879835.1897603803</v>
       </c>
       <c r="AM133">
         <v>0</v>
@@ -16841,16 +16841,16 @@
         <v>1700</v>
       </c>
       <c r="AC135">
-        <v>21946478.87323944</v>
+        <v>39246604.72503889</v>
       </c>
       <c r="AD135">
-        <v>714035.0877192983</v>
+        <v>1191473.335354072</v>
       </c>
       <c r="AE135">
-        <v>7333333.333333333</v>
+        <v>12236753.17390669</v>
       </c>
       <c r="AF135">
-        <v>11429441.64345289</v>
+        <v>19071716.76906865</v>
       </c>
       <c r="AG135">
         <v>0</v>
@@ -16859,16 +16859,16 @@
         <v>5400277.806705137</v>
       </c>
       <c r="AI135">
-        <v>21946478.87323944</v>
+        <v>40061116.44382404</v>
       </c>
       <c r="AJ135">
-        <v>2428842.059390299</v>
+        <v>1216200.799068832</v>
       </c>
       <c r="AK135">
-        <v>13296158.14158557</v>
+        <v>12490710.90935557</v>
       </c>
       <c r="AL135">
-        <v>14292569.37183749</v>
+        <v>19467525.19414362</v>
       </c>
       <c r="AM135">
         <v>0</v>
@@ -17067,16 +17067,16 @@
         <v>394</v>
       </c>
       <c r="AC137">
-        <v>62328767.78531657</v>
+        <v>40622624.70994196</v>
       </c>
       <c r="AD137">
-        <v>168420012.9621428</v>
+        <v>109767338.9560646</v>
       </c>
       <c r="AE137">
-        <v>16570557.0634054</v>
+        <v>10799820.76879713</v>
       </c>
       <c r="AF137">
-        <v>1786744.186046512</v>
+        <v>2098290.697674419</v>
       </c>
       <c r="AG137">
         <v>28579211.93281071</v>
@@ -17085,16 +17085,16 @@
         <v>88669904.66483657</v>
       </c>
       <c r="AI137">
-        <v>63456231.42674965</v>
+        <v>40622624.70994196</v>
       </c>
       <c r="AJ137">
-        <v>172235783.0220167</v>
+        <v>196818927.068079</v>
       </c>
       <c r="AK137">
-        <v>16870301.48754727</v>
+        <v>10321796.60050587</v>
       </c>
       <c r="AL137">
-        <v>1819064.560375875</v>
+        <v>2098290.697674419</v>
       </c>
       <c r="AM137">
         <v>47752648.57910507</v>
@@ -17397,16 +17397,16 @@
         <v>2960</v>
       </c>
       <c r="AC140">
-        <v>17173210.86261981</v>
+        <v>14146177.00611476</v>
       </c>
       <c r="AD140">
-        <v>24786101.01010101</v>
+        <v>20417182.027592</v>
       </c>
       <c r="AE140">
-        <v>3019090.909090909</v>
+        <v>2486931.229064093</v>
       </c>
       <c r="AF140">
-        <v>12453527.27272727</v>
+        <v>11570000</v>
       </c>
       <c r="AG140">
         <v>0</v>
@@ -17415,16 +17415,16 @@
         <v>90294824.7737173</v>
       </c>
       <c r="AI140">
-        <v>17173210.86261981</v>
+        <v>16082104.02126983</v>
       </c>
       <c r="AJ140">
-        <v>103036427.453557</v>
+        <v>101982264.5338659</v>
       </c>
       <c r="AK140">
-        <v>6689656.094043671</v>
+        <v>6621214.402361326</v>
       </c>
       <c r="AL140">
-        <v>19031828.96379587</v>
+        <v>21245540.41651929</v>
       </c>
       <c r="AM140">
         <v>0</v>
@@ -17623,16 +17623,16 @@
         <v>1500</v>
       </c>
       <c r="AC142">
-        <v>2577777.777777778</v>
+        <v>6627908.06359737</v>
       </c>
       <c r="AD142">
-        <v>27293366.33663366</v>
+        <v>36741318.50125522</v>
       </c>
       <c r="AE142">
-        <v>61433200.79522862</v>
+        <v>82699098.71614075</v>
       </c>
       <c r="AF142">
-        <v>10847633.23831251</v>
+        <v>14602681.94395253</v>
       </c>
       <c r="AG142">
         <v>0</v>
@@ -17641,16 +17641,16 @@
         <v>101447765.9677321</v>
       </c>
       <c r="AI142">
-        <v>2577777.777777778</v>
+        <v>6817373.909247481</v>
       </c>
       <c r="AJ142">
-        <v>68430786.08934627</v>
+        <v>61742320.59223025</v>
       </c>
       <c r="AK142">
-        <v>82099893.27466962</v>
+        <v>85063140.96331871</v>
       </c>
       <c r="AL142">
-        <v>10847633.23831251</v>
+        <v>15020115.23613506</v>
       </c>
       <c r="AM142">
         <v>0</v>
@@ -17953,16 +17953,16 @@
         <v>2300</v>
       </c>
       <c r="AC145">
-        <v>7127425.149700599</v>
+        <v>14170000</v>
       </c>
       <c r="AD145">
-        <v>24929432.01376937</v>
+        <v>19420394.94562574</v>
       </c>
       <c r="AE145">
-        <v>31977777.77777778</v>
+        <v>24911160.17344028</v>
       </c>
       <c r="AF145">
-        <v>13116216.21621621</v>
+        <v>10217725.73761199</v>
       </c>
       <c r="AG145">
         <v>0</v>
@@ -17971,16 +17971,16 @@
         <v>6236304.719977756</v>
       </c>
       <c r="AI145">
-        <v>7286279.614384578</v>
+        <v>20054010.39512687</v>
       </c>
       <c r="AJ145">
-        <v>25485053.64349484</v>
+        <v>668839.213889727</v>
       </c>
       <c r="AK145">
-        <v>32690491.3684474</v>
+        <v>35255375.0933551</v>
       </c>
       <c r="AL145">
-        <v>13408547.52267601</v>
+        <v>14460577.14584519</v>
       </c>
       <c r="AM145">
         <v>0</v>
@@ -18387,16 +18387,16 @@
         <v>300</v>
       </c>
       <c r="AC149">
-        <v>14710925.64491654</v>
+        <v>14588302.86311697</v>
       </c>
       <c r="AD149">
-        <v>7343283.582089552</v>
+        <v>7282073.711132854</v>
       </c>
       <c r="AE149">
-        <v>15141612.90322581</v>
+        <v>15015400.13185154</v>
       </c>
       <c r="AF149">
-        <v>956250</v>
+        <v>948279.1871547623</v>
       </c>
       <c r="AG149">
         <v>13648552.25874323</v>
@@ -18405,16 +18405,16 @@
         <v>15350205.64990158</v>
       </c>
       <c r="AI149">
-        <v>14710925.64491654</v>
+        <v>14588302.86311697</v>
       </c>
       <c r="AJ149">
-        <v>28405777.39653199</v>
+        <v>28462892.36801974</v>
       </c>
       <c r="AK149">
-        <v>31220046.31596147</v>
+        <v>31282819.88593953</v>
       </c>
       <c r="AL149">
-        <v>1359857.4987651</v>
+        <v>1362591.739098859</v>
       </c>
       <c r="AM149">
         <v>22805195.6491166</v>
@@ -18509,16 +18509,16 @@
         <v>3000</v>
       </c>
       <c r="AC150">
-        <v>231551120.1629328</v>
+        <v>2441610345.270957</v>
       </c>
       <c r="AD150">
-        <v>2290196.078431372</v>
+        <v>30790186.64722703</v>
       </c>
       <c r="AE150">
-        <v>5334630.350194551</v>
+        <v>56251460.33440147</v>
       </c>
       <c r="AF150">
-        <v>16569150.73583248</v>
+        <v>174714809.5007949</v>
       </c>
       <c r="AG150">
         <v>257629769.0521518</v>
@@ -18527,16 +18527,16 @@
         <v>704518777.5951618</v>
       </c>
       <c r="AI150">
-        <v>2179074550.533812</v>
+        <v>2516971981.614447</v>
       </c>
       <c r="AJ150">
-        <v>94694104.34445441</v>
+        <v>51186684.12428126</v>
       </c>
       <c r="AK150">
-        <v>117570842.4058809</v>
+        <v>49845218.18752873</v>
       </c>
       <c r="AL150">
-        <v>251858200.4240514</v>
+        <v>106777553.8182861</v>
       </c>
       <c r="AM150">
         <v>430470366.1523768</v>
@@ -18631,16 +18631,16 @@
         <v>10</v>
       </c>
       <c r="AC151">
-        <v>1260000</v>
+        <v>565429.7637428906</v>
       </c>
       <c r="AD151">
-        <v>13333.33333333333</v>
+        <v>40000</v>
       </c>
       <c r="AE151">
         <v>0</v>
       </c>
       <c r="AF151">
-        <v>46626.87273695783</v>
+        <v>20923.98542518086</v>
       </c>
       <c r="AG151">
         <v>0</v>
@@ -18649,16 +18649,16 @@
         <v>417569.1661120477</v>
       </c>
       <c r="AI151">
-        <v>1369905.210737807</v>
+        <v>621255.0486534616</v>
       </c>
       <c r="AJ151">
-        <v>14496.3514363789</v>
+        <v>100841.6871419562</v>
       </c>
       <c r="AK151">
         <v>0</v>
       </c>
       <c r="AL151">
-        <v>50693.96501806913</v>
+        <v>19392.33449461724</v>
       </c>
       <c r="AM151">
         <v>0</v>
@@ -18756,10 +18756,10 @@
         <v>0</v>
       </c>
       <c r="AD152">
-        <v>80972580.64516132</v>
+        <v>227004780.7612772</v>
       </c>
       <c r="AE152">
-        <v>63600000</v>
+        <v>178301147.6401545</v>
       </c>
       <c r="AF152">
         <v>0</v>
@@ -18774,10 +18774,10 @@
         <v>0</v>
       </c>
       <c r="AJ152">
-        <v>461730863.0669175</v>
+        <v>461730863.0669174</v>
       </c>
       <c r="AK152">
-        <v>193309440.6270523</v>
+        <v>193309440.6270522</v>
       </c>
       <c r="AL152">
         <v>0</v>
@@ -18961,16 +18961,16 @@
         <v>62.02077895833333</v>
       </c>
       <c r="AC154">
-        <v>3906283.738765371</v>
+        <v>3808728.29985836</v>
       </c>
       <c r="AD154">
-        <v>835996.9712990447</v>
+        <v>1005944.36432331</v>
       </c>
       <c r="AE154">
-        <v>1442902.195454104</v>
+        <v>1449274.631293589</v>
       </c>
       <c r="AF154">
-        <v>3153858.556005829</v>
+        <v>3075094.166049091</v>
       </c>
       <c r="AG154">
         <v>0</v>
@@ -18979,16 +18979,16 @@
         <v>5718882.057621523</v>
       </c>
       <c r="AI154">
-        <v>4613461.705387989</v>
+        <v>4498245.220450297</v>
       </c>
       <c r="AJ154">
-        <v>1342522.275256969</v>
+        <v>1575770.715252568</v>
       </c>
       <c r="AK154">
-        <v>1235090.311513867</v>
+        <v>1210081.936184067</v>
       </c>
       <c r="AL154">
-        <v>3724820.480383723</v>
+        <v>3631796.900655613</v>
       </c>
       <c r="AM154">
         <v>0</v>
@@ -19086,13 +19086,13 @@
         <v>0</v>
       </c>
       <c r="AD155">
-        <v>2206896.551724138</v>
+        <v>9936033.061525501</v>
       </c>
       <c r="AE155">
         <v>0</v>
       </c>
       <c r="AF155">
-        <v>0</v>
+        <v>81837670.55970503</v>
       </c>
       <c r="AG155">
         <v>0</v>
@@ -19104,13 +19104,13 @@
         <v>0</v>
       </c>
       <c r="AJ155">
-        <v>104226413.2490175</v>
+        <v>23533452.80280147</v>
       </c>
       <c r="AK155">
         <v>0</v>
       </c>
       <c r="AL155">
-        <v>0</v>
+        <v>86021934.52012816</v>
       </c>
       <c r="AM155">
         <v>0</v>
@@ -19517,16 +19517,16 @@
         <v>186</v>
       </c>
       <c r="AC159">
-        <v>12975537.84860558</v>
+        <v>10300000</v>
       </c>
       <c r="AD159">
-        <v>77499.99999999999</v>
+        <v>50000</v>
       </c>
       <c r="AE159">
-        <v>1351600</v>
+        <v>1090000</v>
       </c>
       <c r="AF159">
-        <v>983904.6361992406</v>
+        <v>317388.5923223357</v>
       </c>
       <c r="AG159">
         <v>0</v>
@@ -19535,16 +19535,16 @@
         <v>23480821.96953721</v>
       </c>
       <c r="AI159">
-        <v>27249053.76114054</v>
+        <v>28772359.0906895</v>
       </c>
       <c r="AJ159">
-        <v>715077.0356938913</v>
+        <v>613667.7820744767</v>
       </c>
       <c r="AK159">
-        <v>6647285.56414452</v>
+        <v>7130743.936221296</v>
       </c>
       <c r="AL159">
-        <v>3337411.119964842</v>
+        <v>1432056.671958522</v>
       </c>
       <c r="AM159">
         <v>0</v>
@@ -19725,16 +19725,16 @@
         <v>62.82165000000001</v>
       </c>
       <c r="AC161">
-        <v>1194436.914061408</v>
+        <v>1336307.889087182</v>
       </c>
       <c r="AD161">
-        <v>185917.9245668836</v>
+        <v>145101.0733324014</v>
       </c>
       <c r="AE161">
-        <v>295437.7593774619</v>
+        <v>230576.6702616545</v>
       </c>
       <c r="AF161">
-        <v>164856.7610467434</v>
+        <v>128663.726371258</v>
       </c>
       <c r="AG161">
         <v>0</v>
@@ -19743,16 +19743,16 @@
         <v>1089310.868118385</v>
       </c>
       <c r="AI161">
-        <v>1452591.378567107</v>
+        <v>1625125.024141254</v>
       </c>
       <c r="AJ161">
-        <v>264169.1142633214</v>
+        <v>237404.1105990458</v>
       </c>
       <c r="AK161">
-        <v>223754.5126469211</v>
+        <v>201084.2229440777</v>
       </c>
       <c r="AL161">
-        <v>200487.3651976613</v>
+        <v>77389.01299063275</v>
       </c>
       <c r="AM161">
         <v>0</v>
@@ -19847,16 +19847,16 @@
         <v>404</v>
       </c>
       <c r="AC162">
-        <v>5210833.333333333</v>
+        <v>37956820.25258245</v>
       </c>
       <c r="AD162">
-        <v>1094252.873563218</v>
+        <v>6837098.359863644</v>
       </c>
       <c r="AE162">
-        <v>2981103.286862346</v>
+        <v>18626495.65344104</v>
       </c>
       <c r="AF162">
-        <v>2962666.666666667</v>
+        <v>18511300.17281065</v>
       </c>
       <c r="AG162">
         <v>26230000.71193367</v>
@@ -19865,16 +19865,16 @@
         <v>2930111.752415232</v>
       </c>
       <c r="AI162">
-        <v>30880601.98506705</v>
+        <v>37956820.25258245</v>
       </c>
       <c r="AJ162">
-        <v>28491895.49244317</v>
+        <v>26439309.14887551</v>
       </c>
       <c r="AK162">
-        <v>41373827.06325458</v>
+        <v>38393212.7186003</v>
       </c>
       <c r="AL162">
-        <v>28359071.73448219</v>
+        <v>26316054.15518872</v>
       </c>
       <c r="AM162">
         <v>43827380.86590263</v>
@@ -19969,16 +19969,16 @@
         <v>30</v>
       </c>
       <c r="AC163">
-        <v>7883193.277310924</v>
+        <v>5678825.936055198</v>
       </c>
       <c r="AD163">
-        <v>4003053.435114502</v>
+        <v>2883684.67841214</v>
       </c>
       <c r="AE163">
-        <v>608145.0705199186</v>
+        <v>438090.2355004404</v>
       </c>
       <c r="AF163">
-        <v>175000</v>
+        <v>350000</v>
       </c>
       <c r="AG163">
         <v>7140779.40885189</v>
@@ -19987,16 +19987,16 @@
         <v>3676424.179899551</v>
       </c>
       <c r="AI163">
-        <v>9445957.972200848</v>
+        <v>9274612.224176003</v>
       </c>
       <c r="AJ163">
-        <v>21074646.24791316</v>
+        <v>20692360.9321903</v>
       </c>
       <c r="AK163">
-        <v>1706558.268639077</v>
+        <v>1675602.011587277</v>
       </c>
       <c r="AL163">
-        <v>338697.9185988121</v>
+        <v>923285.2393983174</v>
       </c>
       <c r="AM163">
         <v>11931439.20460364</v>
@@ -20091,16 +20091,16 @@
         <v>0</v>
       </c>
       <c r="AC164">
-        <v>67555075.71168989</v>
+        <v>83036382.20107718</v>
       </c>
       <c r="AD164">
-        <v>7771774.193548388</v>
+        <v>9552798.298533788</v>
       </c>
       <c r="AE164">
-        <v>55527238.97911832</v>
+        <v>68252177.79517283</v>
       </c>
       <c r="AF164">
-        <v>0</v>
+        <v>14799317.26591689</v>
       </c>
       <c r="AG164">
         <v>60396756.86648395</v>
@@ -20109,16 +20109,16 @@
         <v>2115078.602263198</v>
       </c>
       <c r="AI164">
-        <v>83911461.23696268</v>
+        <v>83036382.20107718</v>
       </c>
       <c r="AJ164">
-        <v>42413932.84783562</v>
+        <v>38084874.73279537</v>
       </c>
       <c r="AK164">
-        <v>161524897.6110139</v>
+        <v>145038554.0480945</v>
       </c>
       <c r="AL164">
-        <v>0</v>
+        <v>21690480.71384507</v>
       </c>
       <c r="AM164">
         <v>100916187.358257</v>
@@ -20733,16 +20733,16 @@
         <v>4666.5</v>
       </c>
       <c r="AC170">
-        <v>6475123.961661341</v>
+        <v>12132811.73841817</v>
       </c>
       <c r="AD170">
-        <v>16188789.9408284</v>
+        <v>26865438.81259759</v>
       </c>
       <c r="AE170">
-        <v>8801168.83116883</v>
+        <v>14605616.82357637</v>
       </c>
       <c r="AF170">
-        <v>15436996.55172414</v>
+        <v>25617831.0933969</v>
       </c>
       <c r="AG170">
         <v>0</v>
@@ -20751,16 +20751,16 @@
         <v>155683263.6313113</v>
       </c>
       <c r="AI170">
-        <v>13229570.00836878</v>
+        <v>14836840.05032908</v>
       </c>
       <c r="AJ170">
-        <v>145323919.0676158</v>
+        <v>144344076.4904189</v>
       </c>
       <c r="AK170">
-        <v>42112215.50185191</v>
+        <v>41828275.03263289</v>
       </c>
       <c r="AL170">
-        <v>50943771.48222862</v>
+        <v>50600284.48668419</v>
       </c>
       <c r="AM170">
         <v>0</v>
@@ -21479,16 +21479,16 @@
         <v>5100</v>
       </c>
       <c r="AC177">
-        <v>80809107.74930534</v>
+        <v>74570000</v>
       </c>
       <c r="AD177">
-        <v>42482042.25352114</v>
+        <v>27324785.44797364</v>
       </c>
       <c r="AE177">
-        <v>50978643.0223593</v>
+        <v>32789866.23811261</v>
       </c>
       <c r="AF177">
-        <v>25676800</v>
+        <v>16515520.76530351</v>
       </c>
       <c r="AG177">
         <v>0</v>
@@ -21497,16 +21497,16 @@
         <v>168461925.7545083</v>
       </c>
       <c r="AI177">
-        <v>80809107.74930534</v>
+        <v>74570000</v>
       </c>
       <c r="AJ177">
-        <v>102830580.5176575</v>
+        <v>106181647.6728689</v>
       </c>
       <c r="AK177">
-        <v>65773385.50081619</v>
+        <v>67916824.06480438</v>
       </c>
       <c r="AL177">
-        <v>22848798.74499979</v>
+        <v>23593400.77510557</v>
       </c>
       <c r="AM177">
         <v>0</v>
@@ -21705,16 +21705,16 @@
         <v>177.6144178325824</v>
       </c>
       <c r="AC179">
-        <v>27433591.62493549</v>
+        <v>10811911.76470588</v>
       </c>
       <c r="AD179">
-        <v>604777.0927199431</v>
+        <v>238350</v>
       </c>
       <c r="AE179">
         <v>0</v>
       </c>
       <c r="AF179">
-        <v>177614.4178325824</v>
+        <v>70000</v>
       </c>
       <c r="AG179">
         <v>0</v>
@@ -21723,16 +21723,16 @@
         <v>7425469.084340326</v>
       </c>
       <c r="AI179">
-        <v>29424226.14477703</v>
+        <v>11891518.42744402</v>
       </c>
       <c r="AJ179">
-        <v>648660.889418421</v>
+        <v>1151794.627290737</v>
       </c>
       <c r="AK179">
         <v>0</v>
       </c>
       <c r="AL179">
-        <v>190502.4638526934</v>
+        <v>124355.0725312546</v>
       </c>
       <c r="AM179">
         <v>0</v>
@@ -21931,16 +21931,16 @@
         <v>1468</v>
       </c>
       <c r="AC181">
-        <v>11282925.31120332</v>
+        <v>15733347.65557366</v>
       </c>
       <c r="AD181">
-        <v>7429657.568238213</v>
+        <v>8184343.991872499</v>
       </c>
       <c r="AE181">
-        <v>4372954.545454546</v>
+        <v>4817148.560631339</v>
       </c>
       <c r="AF181">
-        <v>4240888.888888889</v>
+        <v>4671667.998045716</v>
       </c>
       <c r="AG181">
         <v>72532873.38702735</v>
@@ -21949,16 +21949,16 @@
         <v>27686651.23134229</v>
       </c>
       <c r="AI181">
-        <v>58281595.03951232</v>
+        <v>70319190.67120777</v>
       </c>
       <c r="AJ181">
-        <v>168617864.5945864</v>
+        <v>160716945.8421294</v>
       </c>
       <c r="AK181">
-        <v>52899890.73428137</v>
+        <v>50421163.22987179</v>
       </c>
       <c r="AL181">
-        <v>35383211.99704006</v>
+        <v>33725262.62221118</v>
       </c>
       <c r="AM181">
         <v>121194273.0060716</v>
@@ -22035,16 +22035,16 @@
         <v>89.49593836999999</v>
       </c>
       <c r="AC182">
-        <v>14172984.41348477</v>
+        <v>13553423.62187831</v>
       </c>
       <c r="AD182">
-        <v>6673356.755619106</v>
+        <v>4486320.380573709</v>
       </c>
       <c r="AE182">
-        <v>9383589.922142759</v>
+        <v>8932832.51589627</v>
       </c>
       <c r="AF182">
-        <v>3780000</v>
+        <v>7037354.572898352</v>
       </c>
       <c r="AG182">
         <v>0</v>
@@ -22053,16 +22053,16 @@
         <v>3991716.481451627</v>
       </c>
       <c r="AI182">
-        <v>14631649.20010926</v>
+        <v>13992038.24052176</v>
       </c>
       <c r="AJ182">
-        <v>6889319.298375659</v>
+        <v>4631506.258159743</v>
       </c>
       <c r="AK182">
-        <v>9687260.775355328</v>
+        <v>9221916.000385089</v>
       </c>
       <c r="AL182">
-        <v>3902328.003958787</v>
+        <v>7265096.778732451</v>
       </c>
       <c r="AM182">
         <v>0</v>
@@ -22157,16 +22157,16 @@
         <v>15200</v>
       </c>
       <c r="AC183">
-        <v>291195627.8959249</v>
+        <v>258750126.6484495</v>
       </c>
       <c r="AD183">
-        <v>733059812.9261283</v>
+        <v>607321117.1682</v>
       </c>
       <c r="AE183">
-        <v>572436173.6859288</v>
+        <v>474248581.6030699</v>
       </c>
       <c r="AF183">
-        <v>71405974.00207794</v>
+        <v>66120052.82134517</v>
       </c>
       <c r="AG183">
         <v>964610824.0639657</v>
@@ -22175,16 +22175,16 @@
         <v>2317082225.165185</v>
       </c>
       <c r="AI183">
-        <v>430310925.5049419</v>
+        <v>458327893.6901452</v>
       </c>
       <c r="AJ183">
-        <v>4759507398.057753</v>
+        <v>4726494664.514017</v>
       </c>
       <c r="AK183">
-        <v>1981046589.145263</v>
+        <v>1967305721.08571</v>
       </c>
       <c r="AL183">
-        <v>170436542.3180736</v>
+        <v>189173175.7361592</v>
       </c>
       <c r="AM183">
         <v>1611756188.568819</v>
@@ -22279,13 +22279,13 @@
         <v>0</v>
       </c>
       <c r="AC184">
-        <v>10537815.12605042</v>
+        <v>9532503.54879483</v>
       </c>
       <c r="AD184">
-        <v>4787234.042553192</v>
+        <v>4330530.091265085</v>
       </c>
       <c r="AE184">
-        <v>11924413.14744939</v>
+        <v>10786819.59074759</v>
       </c>
       <c r="AF184">
         <v>0</v>
@@ -22300,7 +22300,7 @@
         <v>19470111.42779673</v>
       </c>
       <c r="AJ184">
-        <v>38862218.90627506</v>
+        <v>38862218.90627505</v>
       </c>
       <c r="AK184">
         <v>51597061.97087712</v>
@@ -22609,16 +22609,16 @@
         <v>4881</v>
       </c>
       <c r="AC187">
-        <v>129719790.8055672</v>
+        <v>88720000</v>
       </c>
       <c r="AD187">
-        <v>101689221.2104981</v>
+        <v>24756015.27307653</v>
       </c>
       <c r="AE187">
-        <v>113596723.3009709</v>
+        <v>27654870.23633495</v>
       </c>
       <c r="AF187">
-        <v>11970071.42857143</v>
+        <v>2914087.329788094</v>
       </c>
       <c r="AG187">
         <v>0</v>
@@ -22627,16 +22627,16 @@
         <v>162433692.7761187</v>
       </c>
       <c r="AI187">
-        <v>198525027.3241806</v>
+        <v>88720000</v>
       </c>
       <c r="AJ187">
-        <v>11069000.1897571</v>
+        <v>106058512.3011746</v>
       </c>
       <c r="AK187">
-        <v>173850053.6981653</v>
+        <v>63151175.42934998</v>
       </c>
       <c r="AL187">
-        <v>18319168.89992046</v>
+        <v>4589579.791311916</v>
       </c>
       <c r="AM187">
         <v>0</v>
@@ -22939,16 +22939,16 @@
         <v>25.47</v>
       </c>
       <c r="AC190">
-        <v>178290</v>
+        <v>780727.8344024753</v>
       </c>
       <c r="AD190">
-        <v>318375</v>
+        <v>1183639.163228038</v>
       </c>
       <c r="AE190">
-        <v>491207.142857143</v>
+        <v>1826186.137551831</v>
       </c>
       <c r="AF190">
-        <v>118758.6448610316</v>
+        <v>441515.141042504</v>
       </c>
       <c r="AG190">
         <v>0</v>
@@ -22957,16 +22957,16 @@
         <v>5609950.970809684</v>
       </c>
       <c r="AI190">
-        <v>553722.6653866367</v>
+        <v>780727.8344024753</v>
       </c>
       <c r="AJ190">
-        <v>4344395.402540626</v>
+        <v>4228547.263558079</v>
       </c>
       <c r="AK190">
-        <v>3572729.084271279</v>
+        <v>3477458.286576483</v>
       </c>
       <c r="AL190">
-        <v>595746.080525747</v>
+        <v>579859.8481872509</v>
       </c>
       <c r="AM190">
         <v>0</v>
@@ -23165,16 +23165,16 @@
         <v>0</v>
       </c>
       <c r="AC192">
-        <v>6746666.666666668</v>
+        <v>7357691.867689863</v>
       </c>
       <c r="AD192">
-        <v>24665187.40629686</v>
+        <v>26899038.85291849</v>
       </c>
       <c r="AE192">
-        <v>57248895.3488372</v>
+        <v>62433754.70489635</v>
       </c>
       <c r="AF192">
-        <v>0</v>
+        <v>712467.4057057982</v>
       </c>
       <c r="AG192">
         <v>9145831.341171443</v>
@@ -23183,16 +23183,16 @@
         <v>193152609.1544196</v>
       </c>
       <c r="AI192">
-        <v>9374995.415789433</v>
+        <v>9335463.197948266</v>
       </c>
       <c r="AJ192">
-        <v>150588324.7319508</v>
+        <v>149953328.105967</v>
       </c>
       <c r="AK192">
-        <v>186302643.7866955</v>
+        <v>185517048.0213731</v>
       </c>
       <c r="AL192">
-        <v>0</v>
+        <v>1460124.609147463</v>
       </c>
       <c r="AM192">
         <v>15281655.45731242</v>

</xml_diff>